<commit_message>
Mixtos: "Inicio de construcción" pasa a "Inicio de inversión"
- Excel DATOS_MIXTOS.xlsx: se renombra el encabezado de la columna y la
  nota de la hoja "Instrucciones" (solo el texto dentro del archivo; el
  formato y la fecha de guardado no cambian, así que no se crea un corte
  nuevo).
- Ficha: la etiqueta dice "Inicio de inversión"; el campo interno pasa a
  inicioInversion.
- Validación (data-rules.js): la columna obligatoria y de fecha ahora es
  "Inicio de Inversión". DATOS_MIXTOS.json regenerado.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01APiq7bAy76yveceNZKtsYf
</commit_message>
<xml_diff>
--- a/cartera-mixtos/data/DATOS_MIXTOS.xlsx
+++ b/cartera-mixtos/data/DATOS_MIXTOS.xlsx
@@ -66,7 +66,7 @@
     <t>Horas de Almacenamiento</t>
   </si>
   <si>
-    <t>Inicio de Construcción</t>
+    <t>Inicio de Inversión</t>
   </si>
   <si>
     <t>Fin de Construcción</t>
@@ -135,7 +135,7 @@
     <t xml:space="preserve">   uses el formato de porcentaje de Excel (para evitar que 92 se vuelva 9200%).</t>
   </si>
   <si>
-    <t>• Fechas (Inicio de Construcción, Fin de Construcción, Fecha firma de contrato):</t>
+    <t>• Fechas (Inicio de Inversión, Fin de Construcción, Fecha firma de contrato):</t>
   </si>
   <si>
     <t xml:space="preserve">   escribe el formato AAAA-MM-DD como texto, ej. 2024-03-01. Esas columnas ya</t>

</xml_diff>

<commit_message>
Mixtos: Concepción Mendizábal se divide en Fase I, II y III
- Excel: la fila del proyecto combinado se sustituye por tres filas (una
  por fase) con su capacidad, almacenamiento, CAPEX y avances al 30-sep-26;
  socio, tecnología, ubicación y fechas compartidas. Se editó solo la hoja
  Proyectos para conservar el formato.
- KML (del usuario): un punto y sus polígonos por fase.
- Historial: las tres fases ocupan el lugar del proyecto combinado en los
  cortes existentes, con sus avances del 21-sep-26 (corte del 25 sep) y del
  30-sep-26 (cortes del 2 y 5 oct).
- Esta semana: se quitan las entradas del proyecto combinado; las fases
  no aparecen como cambios.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01APiq7bAy76yveceNZKtsYf
</commit_message>
<xml_diff>
--- a/cartera-mixtos/data/DATOS_MIXTOS.xlsx
+++ b/cartera-mixtos/data/DATOS_MIXTOS.xlsx
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="642" uniqueCount="356">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="657" uniqueCount="366">
   <si>
     <t>NO.</t>
   </si>
@@ -1105,6 +1105,36 @@
   </si>
   <si>
     <t>53.60%</t>
+  </si>
+  <si>
+    <t>CONCEPCIÓN MENDIZÁBAL MENDOZA FASE I</t>
+  </si>
+  <si>
+    <t>339 MW</t>
+  </si>
+  <si>
+    <t>101.7 MW / 305.1 MWh</t>
+  </si>
+  <si>
+    <t>$381,545,675.00</t>
+  </si>
+  <si>
+    <t>CONCEPCIÓN MENDIZÁBAL MENDOZA FASE II</t>
+  </si>
+  <si>
+    <t>180 MW</t>
+  </si>
+  <si>
+    <t>54 MW / 162 MWh</t>
+  </si>
+  <si>
+    <t>$198,977,154.00</t>
+  </si>
+  <si>
+    <t>CONCEPCIÓN MENDIZÁBAL MENDOZA FASE III</t>
+  </si>
+  <si>
+    <t>$376,737,492.00</t>
   </si>
 </sst>
 </file>
@@ -1486,7 +1516,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q40"/>
+  <dimension ref="A1:Q42"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4.85546875" bestFit="1" customWidth="1"/>
@@ -3155,10 +3185,10 @@
         <v>31</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>166</v>
+        <v>356</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>166</v>
+        <v>356</v>
       </c>
       <c r="D32" s="6" t="s">
         <v>167</v>
@@ -3170,10 +3200,10 @@
         <v>168</v>
       </c>
       <c r="G32" s="6" t="s">
-        <v>321</v>
+        <v>357</v>
       </c>
       <c r="H32" s="6" t="s">
-        <v>322</v>
+        <v>358</v>
       </c>
       <c r="I32" s="6" t="s">
         <v>189</v>
@@ -3188,16 +3218,16 @@
         <v>325</v>
       </c>
       <c r="M32" s="6" t="s">
-        <v>265</v>
+        <v>359</v>
       </c>
       <c r="N32" s="6" t="s">
-        <v>343</v>
+        <v>328</v>
       </c>
       <c r="O32" s="6" t="s">
-        <v>343</v>
+        <v>328</v>
       </c>
       <c r="P32" s="6" t="s">
-        <v>343</v>
+        <v>328</v>
       </c>
       <c r="Q32" s="6" t="s">
         <v>296</v>
@@ -3208,49 +3238,49 @@
         <v>32</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>163</v>
+        <v>360</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>163</v>
+        <v>360</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="E33" s="6" t="s">
         <v>40</v>
       </c>
       <c r="F33" s="6" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="G33" s="6" t="s">
-        <v>323</v>
+        <v>361</v>
       </c>
       <c r="H33" s="6" t="s">
-        <v>324</v>
+        <v>362</v>
       </c>
       <c r="I33" s="6" t="s">
         <v>189</v>
       </c>
       <c r="J33" s="6" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="K33" s="6" t="s">
-        <v>227</v>
+        <v>202</v>
       </c>
       <c r="L33" s="6" t="s">
-        <v>224</v>
+        <v>325</v>
       </c>
       <c r="M33" s="6" t="s">
-        <v>344</v>
+        <v>363</v>
       </c>
       <c r="N33" s="6" t="s">
         <v>328</v>
       </c>
       <c r="O33" s="6" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="P33" s="6" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="Q33" s="6" t="s">
         <v>296</v>
@@ -3261,52 +3291,52 @@
         <v>33</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>170</v>
+        <v>364</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>170</v>
+        <v>364</v>
       </c>
       <c r="D34" s="6" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="E34" s="6" t="s">
         <v>40</v>
       </c>
       <c r="F34" s="6" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="G34" s="6" t="s">
-        <v>173</v>
+        <v>357</v>
       </c>
       <c r="H34" s="6" t="s">
-        <v>174</v>
+        <v>358</v>
       </c>
       <c r="I34" s="6" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="J34" s="6" t="s">
-        <v>231</v>
+        <v>201</v>
       </c>
       <c r="K34" s="6" t="s">
-        <v>232</v>
+        <v>202</v>
       </c>
       <c r="L34" s="6" t="s">
-        <v>169</v>
+        <v>325</v>
       </c>
       <c r="M34" s="6" t="s">
-        <v>344</v>
+        <v>365</v>
       </c>
       <c r="N34" s="6" t="s">
-        <v>278</v>
+        <v>285</v>
       </c>
       <c r="O34" s="6" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="P34" s="6" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
       <c r="Q34" s="6" t="s">
-        <v>20</v>
+        <v>296</v>
       </c>
     </row>
     <row r="35" spans="1:17" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -3314,52 +3344,52 @@
         <v>34</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>175</v>
+        <v>163</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>175</v>
+        <v>163</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>176</v>
+        <v>164</v>
       </c>
       <c r="E35" s="6" t="s">
         <v>40</v>
       </c>
       <c r="F35" s="6" t="s">
-        <v>152</v>
+        <v>165</v>
       </c>
       <c r="G35" s="6" t="s">
-        <v>118</v>
+        <v>323</v>
       </c>
       <c r="H35" s="6" t="s">
-        <v>177</v>
+        <v>324</v>
       </c>
       <c r="I35" s="6" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="J35" s="6" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="K35" s="6" t="s">
-        <v>221</v>
+        <v>227</v>
       </c>
       <c r="L35" s="6" t="s">
-        <v>169</v>
+        <v>224</v>
       </c>
       <c r="M35" s="6" t="s">
         <v>344</v>
       </c>
       <c r="N35" s="6" t="s">
-        <v>276</v>
+        <v>328</v>
       </c>
       <c r="O35" s="6" t="s">
-        <v>270</v>
+        <v>329</v>
       </c>
       <c r="P35" s="6" t="s">
-        <v>290</v>
+        <v>330</v>
       </c>
       <c r="Q35" s="6" t="s">
-        <v>20</v>
+        <v>296</v>
       </c>
     </row>
     <row r="36" spans="1:17" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -3367,34 +3397,34 @@
         <v>35</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>19</v>
+        <v>170</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>19</v>
+        <v>170</v>
       </c>
       <c r="D36" s="6" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="E36" s="6" t="s">
         <v>40</v>
       </c>
       <c r="F36" s="6" t="s">
-        <v>152</v>
+        <v>172</v>
       </c>
       <c r="G36" s="6" t="s">
-        <v>118</v>
+        <v>173</v>
       </c>
       <c r="H36" s="6" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="I36" s="6" t="s">
         <v>187</v>
       </c>
       <c r="J36" s="6" t="s">
-        <v>206</v>
+        <v>231</v>
       </c>
       <c r="K36" s="6" t="s">
-        <v>221</v>
+        <v>232</v>
       </c>
       <c r="L36" s="6" t="s">
         <v>169</v>
@@ -3403,13 +3433,13 @@
         <v>344</v>
       </c>
       <c r="N36" s="6" t="s">
-        <v>291</v>
+        <v>278</v>
       </c>
       <c r="O36" s="6" t="s">
-        <v>270</v>
+        <v>288</v>
       </c>
       <c r="P36" s="6" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="Q36" s="6" t="s">
         <v>20</v>
@@ -3420,10 +3450,10 @@
         <v>36</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="D37" s="6" t="s">
         <v>176</v>
@@ -3456,13 +3486,13 @@
         <v>344</v>
       </c>
       <c r="N37" s="6" t="s">
-        <v>293</v>
+        <v>276</v>
       </c>
       <c r="O37" s="6" t="s">
         <v>270</v>
       </c>
       <c r="P37" s="6" t="s">
-        <v>294</v>
+        <v>290</v>
       </c>
       <c r="Q37" s="6" t="s">
         <v>20</v>
@@ -3473,34 +3503,34 @@
         <v>37</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>179</v>
+        <v>19</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>179</v>
+        <v>19</v>
       </c>
       <c r="D38" s="6" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="F38" s="6" t="s">
-        <v>181</v>
+        <v>152</v>
       </c>
       <c r="G38" s="6" t="s">
-        <v>182</v>
+        <v>118</v>
       </c>
       <c r="H38" s="6" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
       <c r="I38" s="6" t="s">
         <v>187</v>
       </c>
       <c r="J38" s="6" t="s">
-        <v>233</v>
+        <v>206</v>
       </c>
       <c r="K38" s="6" t="s">
-        <v>234</v>
+        <v>221</v>
       </c>
       <c r="L38" s="6" t="s">
         <v>169</v>
@@ -3509,13 +3539,13 @@
         <v>344</v>
       </c>
       <c r="N38" s="6" t="s">
-        <v>295</v>
+        <v>291</v>
       </c>
       <c r="O38" s="6" t="s">
-        <v>295</v>
+        <v>270</v>
       </c>
       <c r="P38" s="6" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="Q38" s="6" t="s">
         <v>20</v>
@@ -3526,34 +3556,34 @@
         <v>38</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
       <c r="D39" s="6" t="s">
-        <v>65</v>
+        <v>176</v>
       </c>
       <c r="E39" s="6" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="F39" s="6" t="s">
-        <v>70</v>
+        <v>152</v>
       </c>
       <c r="G39" s="6" t="s">
-        <v>185</v>
+        <v>118</v>
       </c>
       <c r="H39" s="6" t="s">
-        <v>186</v>
+        <v>177</v>
       </c>
       <c r="I39" s="6" t="s">
         <v>187</v>
       </c>
       <c r="J39" s="6" t="s">
-        <v>228</v>
+        <v>206</v>
       </c>
       <c r="K39" s="6" t="s">
-        <v>211</v>
+        <v>221</v>
       </c>
       <c r="L39" s="6" t="s">
         <v>169</v>
@@ -3562,22 +3592,128 @@
         <v>344</v>
       </c>
       <c r="N39" s="6" t="s">
+        <v>293</v>
+      </c>
+      <c r="O39" s="6" t="s">
+        <v>270</v>
+      </c>
+      <c r="P39" s="6" t="s">
+        <v>294</v>
+      </c>
+      <c r="Q39" s="6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="40" spans="1:17" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="2">
+        <v>39</v>
+      </c>
+      <c r="B40" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="C40" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="D40" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="E40" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="F40" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="G40" s="6" t="s">
+        <v>182</v>
+      </c>
+      <c r="H40" s="6" t="s">
+        <v>183</v>
+      </c>
+      <c r="I40" s="6" t="s">
+        <v>187</v>
+      </c>
+      <c r="J40" s="6" t="s">
+        <v>233</v>
+      </c>
+      <c r="K40" s="6" t="s">
+        <v>234</v>
+      </c>
+      <c r="L40" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="M40" s="6" t="s">
+        <v>344</v>
+      </c>
+      <c r="N40" s="6" t="s">
+        <v>295</v>
+      </c>
+      <c r="O40" s="6" t="s">
+        <v>295</v>
+      </c>
+      <c r="P40" s="6" t="s">
+        <v>295</v>
+      </c>
+      <c r="Q40" s="6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="41" spans="1:17" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="2">
+        <v>40</v>
+      </c>
+      <c r="B41" s="6" t="s">
+        <v>184</v>
+      </c>
+      <c r="C41" s="6" t="s">
+        <v>184</v>
+      </c>
+      <c r="D41" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="E41" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="F41" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="G41" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="H41" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="I41" s="6" t="s">
+        <v>187</v>
+      </c>
+      <c r="J41" s="6" t="s">
+        <v>228</v>
+      </c>
+      <c r="K41" s="6" t="s">
+        <v>211</v>
+      </c>
+      <c r="L41" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="M41" s="6" t="s">
+        <v>344</v>
+      </c>
+      <c r="N41" s="6" t="s">
         <v>272</v>
       </c>
-      <c r="O39" s="6" t="s">
+      <c r="O41" s="6" t="s">
         <v>266</v>
       </c>
-      <c r="P39" s="6" t="s">
+      <c r="P41" s="6" t="s">
         <v>273</v>
       </c>
-      <c r="Q39" s="6" t="s">
+      <c r="Q41" s="6" t="s">
         <v>296</v>
       </c>
     </row>
-    <row r="40" spans="1:17" s="6" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="42" spans="1:17" s="6" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <autoFilter ref="A1:Q1" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:Q39">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:Q41">
       <sortCondition ref="A1"/>
     </sortState>
   </autoFilter>

</xml_diff>

<commit_message>
Mixtos: avances de Concepción Mendizábal al 5-oct-26 por fase
Fase I y II: 83.50 %; Fase III: 82.50 % (Parque, LT y Global). Se
actualizan el Excel y los cortes del 2 y 5 de octubre del historial (el
proyecto combinado ya estaba en 83.5 % desde el 2 de octubre). No se
agrega nada a "Esta semana".

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01APiq7bAy76yveceNZKtsYf
</commit_message>
<xml_diff>
--- a/cartera-mixtos/data/DATOS_MIXTOS.xlsx
+++ b/cartera-mixtos/data/DATOS_MIXTOS.xlsx
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="657" uniqueCount="366">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="657" uniqueCount="367">
   <si>
     <t>NO.</t>
   </si>
@@ -1135,6 +1135,9 @@
   </si>
   <si>
     <t>$376,737,492.00</t>
+  </si>
+  <si>
+    <t>82.50%</t>
   </si>
 </sst>
 </file>
@@ -3221,13 +3224,13 @@
         <v>359</v>
       </c>
       <c r="N32" s="6" t="s">
-        <v>328</v>
+        <v>343</v>
       </c>
       <c r="O32" s="6" t="s">
-        <v>328</v>
+        <v>343</v>
       </c>
       <c r="P32" s="6" t="s">
-        <v>328</v>
+        <v>343</v>
       </c>
       <c r="Q32" s="6" t="s">
         <v>296</v>
@@ -3274,13 +3277,13 @@
         <v>363</v>
       </c>
       <c r="N33" s="6" t="s">
-        <v>328</v>
+        <v>343</v>
       </c>
       <c r="O33" s="6" t="s">
-        <v>328</v>
+        <v>343</v>
       </c>
       <c r="P33" s="6" t="s">
-        <v>328</v>
+        <v>343</v>
       </c>
       <c r="Q33" s="6" t="s">
         <v>296</v>
@@ -3327,13 +3330,13 @@
         <v>365</v>
       </c>
       <c r="N34" s="6" t="s">
-        <v>285</v>
+        <v>366</v>
       </c>
       <c r="O34" s="6" t="s">
-        <v>285</v>
+        <v>366</v>
       </c>
       <c r="P34" s="6" t="s">
-        <v>285</v>
+        <v>366</v>
       </c>
       <c r="Q34" s="6" t="s">
         <v>296</v>

</xml_diff>

<commit_message>
Mixtos: proyectos prioritarios (columna PRIORI)
- Excel: nueva columna PRIORI ("P" / "NoP") con los 12 prioritarios y
  su indicación en la hoja Instrucciones. Sin cambiar la fecha del Excel,
  así que no se crea un corte nuevo.
- El ranking del Resumen ahora es "Ranking de proyectos prioritarios":
  todos los prioritarios (de los filtrados) por avance de Parque.
- Tarjetas prioritarias con fondo verde azulado claro, franja lateral y
  distintivo "★ Prioritario" (también en la ficha).
- La validación exige la columna PRIORI con valores P o NoP.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01APiq7bAy76yveceNZKtsYf
</commit_message>
<xml_diff>
--- a/cartera-mixtos/data/DATOS_MIXTOS.xlsx
+++ b/cartera-mixtos/data/DATOS_MIXTOS.xlsx
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="633" uniqueCount="361">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="675" uniqueCount="365">
   <si>
     <t>NO.</t>
   </si>
@@ -1120,6 +1120,18 @@
   </si>
   <si>
     <t>82.75%</t>
+  </si>
+  <si>
+    <t>PRIORI</t>
+  </si>
+  <si>
+    <t>P</t>
+  </si>
+  <si>
+    <t>NoP</t>
+  </si>
+  <si>
+    <t>• PRIORI: escribe "P" si el proyecto es prioritario (aparece en el ranking del Resumen y su tarjeta se distingue) o "NoP" si no lo es.</t>
   </si>
 </sst>
 </file>
@@ -1582,6 +1594,9 @@
       <c r="P1" s="6" t="s">
         <v>15</v>
       </c>
+      <c r="Q1" s="6" t="s">
+        <v>361</v>
+      </c>
     </row>
     <row r="2" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
@@ -1632,7 +1647,9 @@
       <c r="P2" s="1" t="s">
         <v>274</v>
       </c>
-      <c r="Q2"/>
+      <c r="Q2" s="1" t="s">
+        <v>362</v>
+      </c>
     </row>
     <row r="3" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
@@ -1683,6 +1700,9 @@
       <c r="P3" s="1" t="s">
         <v>276</v>
       </c>
+      <c r="Q3" s="1" t="s">
+        <v>363</v>
+      </c>
     </row>
     <row r="4" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
@@ -1733,6 +1753,9 @@
       <c r="P4" s="5" t="s">
         <v>267</v>
       </c>
+      <c r="Q4" s="5" t="s">
+        <v>363</v>
+      </c>
     </row>
     <row r="5" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
@@ -1783,6 +1806,9 @@
       <c r="P5" s="5" t="s">
         <v>295</v>
       </c>
+      <c r="Q5" s="5" t="s">
+        <v>362</v>
+      </c>
     </row>
     <row r="6" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
@@ -1833,6 +1859,9 @@
       <c r="P6" s="5" t="s">
         <v>282</v>
       </c>
+      <c r="Q6" s="5" t="s">
+        <v>362</v>
+      </c>
     </row>
     <row r="7" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
@@ -1883,6 +1912,9 @@
       <c r="P7" s="5" t="s">
         <v>351</v>
       </c>
+      <c r="Q7" s="5" t="s">
+        <v>363</v>
+      </c>
     </row>
     <row r="8" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
@@ -1933,6 +1965,9 @@
       <c r="P8" s="5" t="s">
         <v>351</v>
       </c>
+      <c r="Q8" s="5" t="s">
+        <v>363</v>
+      </c>
     </row>
     <row r="9" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
@@ -1983,6 +2018,9 @@
       <c r="P9" s="5" t="s">
         <v>293</v>
       </c>
+      <c r="Q9" s="5" t="s">
+        <v>363</v>
+      </c>
     </row>
     <row r="10" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
@@ -2033,6 +2071,9 @@
       <c r="P10" s="5" t="s">
         <v>261</v>
       </c>
+      <c r="Q10" s="5" t="s">
+        <v>363</v>
+      </c>
     </row>
     <row r="11" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
@@ -2083,6 +2124,9 @@
       <c r="P11" s="5" t="s">
         <v>292</v>
       </c>
+      <c r="Q11" s="5" t="s">
+        <v>362</v>
+      </c>
     </row>
     <row r="12" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
@@ -2133,6 +2177,9 @@
       <c r="P12" s="5" t="s">
         <v>277</v>
       </c>
+      <c r="Q12" s="5" t="s">
+        <v>362</v>
+      </c>
     </row>
     <row r="13" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
@@ -2183,6 +2230,9 @@
       <c r="P13" s="5" t="s">
         <v>280</v>
       </c>
+      <c r="Q13" s="5" t="s">
+        <v>363</v>
+      </c>
     </row>
     <row r="14" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
@@ -2233,6 +2283,9 @@
       <c r="P14" s="5" t="s">
         <v>300</v>
       </c>
+      <c r="Q14" s="5" t="s">
+        <v>363</v>
+      </c>
     </row>
     <row r="15" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
@@ -2283,6 +2336,9 @@
       <c r="P15" s="5" t="s">
         <v>318</v>
       </c>
+      <c r="Q15" s="5" t="s">
+        <v>363</v>
+      </c>
     </row>
     <row r="16" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
@@ -2333,6 +2389,9 @@
       <c r="P16" s="5" t="s">
         <v>320</v>
       </c>
+      <c r="Q16" s="5" t="s">
+        <v>363</v>
+      </c>
     </row>
     <row r="17" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
@@ -2383,6 +2442,9 @@
       <c r="P17" s="5" t="s">
         <v>326</v>
       </c>
+      <c r="Q17" s="5" t="s">
+        <v>363</v>
+      </c>
     </row>
     <row r="18" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
@@ -2433,6 +2495,9 @@
       <c r="P18" s="5" t="s">
         <v>305</v>
       </c>
+      <c r="Q18" s="5" t="s">
+        <v>362</v>
+      </c>
     </row>
     <row r="19" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
@@ -2483,6 +2548,9 @@
       <c r="P19" s="5" t="s">
         <v>308</v>
       </c>
+      <c r="Q19" s="5" t="s">
+        <v>363</v>
+      </c>
     </row>
     <row r="20" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
@@ -2533,6 +2601,9 @@
       <c r="P20" s="5" t="s">
         <v>309</v>
       </c>
+      <c r="Q20" s="5" t="s">
+        <v>363</v>
+      </c>
     </row>
     <row r="21" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
@@ -2583,6 +2654,9 @@
       <c r="P21" s="5" t="s">
         <v>311</v>
       </c>
+      <c r="Q21" s="5" t="s">
+        <v>363</v>
+      </c>
     </row>
     <row r="22" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
@@ -2633,6 +2707,9 @@
       <c r="P22" s="5" t="s">
         <v>312</v>
       </c>
+      <c r="Q22" s="5" t="s">
+        <v>363</v>
+      </c>
     </row>
     <row r="23" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
@@ -2683,6 +2760,9 @@
       <c r="P23" s="5" t="s">
         <v>315</v>
       </c>
+      <c r="Q23" s="5" t="s">
+        <v>362</v>
+      </c>
     </row>
     <row r="24" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
@@ -2733,6 +2813,9 @@
       <c r="P24" s="5" t="s">
         <v>283</v>
       </c>
+      <c r="Q24" s="5" t="s">
+        <v>362</v>
+      </c>
     </row>
     <row r="25" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
@@ -2783,6 +2866,9 @@
       <c r="P25" s="5" t="s">
         <v>323</v>
       </c>
+      <c r="Q25" s="5" t="s">
+        <v>362</v>
+      </c>
     </row>
     <row r="26" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
@@ -2833,6 +2919,9 @@
       <c r="P26" s="5" t="s">
         <v>324</v>
       </c>
+      <c r="Q26" s="5" t="s">
+        <v>363</v>
+      </c>
     </row>
     <row r="27" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
@@ -2883,6 +2972,9 @@
       <c r="P27" s="5" t="s">
         <v>354</v>
       </c>
+      <c r="Q27" s="5" t="s">
+        <v>362</v>
+      </c>
     </row>
     <row r="28" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
@@ -2933,6 +3025,9 @@
       <c r="P28" s="5" t="s">
         <v>356</v>
       </c>
+      <c r="Q28" s="5" t="s">
+        <v>363</v>
+      </c>
     </row>
     <row r="29" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
@@ -2983,6 +3078,9 @@
       <c r="P29" s="5" t="s">
         <v>357</v>
       </c>
+      <c r="Q29" s="5" t="s">
+        <v>362</v>
+      </c>
     </row>
     <row r="30" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
@@ -3033,6 +3131,9 @@
       <c r="P30" s="5" t="s">
         <v>286</v>
       </c>
+      <c r="Q30" s="5" t="s">
+        <v>363</v>
+      </c>
     </row>
     <row r="31" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
@@ -3083,6 +3184,9 @@
       <c r="P31" s="5" t="s">
         <v>289</v>
       </c>
+      <c r="Q31" s="5" t="s">
+        <v>362</v>
+      </c>
     </row>
     <row r="32" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
@@ -3133,6 +3237,9 @@
       <c r="P32" s="5" t="s">
         <v>359</v>
       </c>
+      <c r="Q32" s="5" t="s">
+        <v>363</v>
+      </c>
     </row>
     <row r="33" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
@@ -3183,6 +3290,9 @@
       <c r="P33" s="5" t="s">
         <v>359</v>
       </c>
+      <c r="Q33" s="5" t="s">
+        <v>363</v>
+      </c>
     </row>
     <row r="34" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
@@ -3233,6 +3343,9 @@
       <c r="P34" s="5" t="s">
         <v>360</v>
       </c>
+      <c r="Q34" s="5" t="s">
+        <v>363</v>
+      </c>
     </row>
     <row r="35" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
@@ -3283,6 +3396,9 @@
       <c r="P35" s="5" t="s">
         <v>303</v>
       </c>
+      <c r="Q35" s="5" t="s">
+        <v>363</v>
+      </c>
     </row>
     <row r="36" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
@@ -3333,6 +3449,9 @@
       <c r="P36" s="5" t="s">
         <v>344</v>
       </c>
+      <c r="Q36" s="5" t="s">
+        <v>363</v>
+      </c>
     </row>
     <row r="37" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
@@ -3383,6 +3502,9 @@
       <c r="P37" s="5" t="s">
         <v>338</v>
       </c>
+      <c r="Q37" s="5" t="s">
+        <v>363</v>
+      </c>
     </row>
     <row r="38" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="1">
@@ -3433,6 +3555,9 @@
       <c r="P38" s="5" t="s">
         <v>338</v>
       </c>
+      <c r="Q38" s="5" t="s">
+        <v>363</v>
+      </c>
     </row>
     <row r="39" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="1">
@@ -3483,6 +3608,9 @@
       <c r="P39" s="5" t="s">
         <v>341</v>
       </c>
+      <c r="Q39" s="5" t="s">
+        <v>363</v>
+      </c>
     </row>
     <row r="40" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="1">
@@ -3533,6 +3661,9 @@
       <c r="P40" s="5" t="s">
         <v>346</v>
       </c>
+      <c r="Q40" s="5" t="s">
+        <v>363</v>
+      </c>
     </row>
     <row r="41" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="1">
@@ -3583,11 +3714,14 @@
       <c r="P41" s="5" t="s">
         <v>358</v>
       </c>
+      <c r="Q41" s="5" t="s">
+        <v>363</v>
+      </c>
     </row>
     <row r="42" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <autoFilter ref="A1:P1" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:P41">
+  <autoFilter ref="A1:Q1" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:Q41">
       <sortCondition ref="A1"/>
     </sortState>
   </autoFilter>
@@ -3597,7 +3731,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:A20"/>
+  <dimension ref="A1:A21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="100" customWidth="1"/>
@@ -3685,15 +3819,20 @@
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" s="3"/>
+      <c r="A18" s="3" t="s">
+        <v>364</v>
+      </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19" s="3" t="s">
-        <v>33</v>
-      </c>
+      <c r="A19" s="3"/>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
         <v>34</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Mixtos: desglose de trámites y permisos por proyecto
- DATOS_MIXTOS.xlsx trae el desglose copiado de "Base de Datos"
  (name_BD + DI_P … AFAC_LT). Revisado contra el Excel de Estado de
  Proyectos: los 40 proyectos coinciden celda por celda y la ponderación
  da exactamente sus Parque, LT y Global.
- tramites.js: trámites, pesos (fila 52 de Base de Datos) y cálculo.
- Ficha: sección "Trámites y permisos" con los 10 trámites agrupados, su
  peso, barras de Parque y LT, y los puntos que faltan.
- Resumen: tarjeta "Trámites más rezagados" (promedio de los proyectos
  mostrados).
- Action "Datos": exige las columnas de trámites y avisa si Parque, LT o
  Global no cuadran con la ponderación. Se quitan del JSON las columnas
  sin encabezado (__EMPTY).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01APiq7bAy76yveceNZKtsYf
</commit_message>
<xml_diff>
--- a/cartera-mixtos/data/DATOS_MIXTOS.xlsx
+++ b/cartera-mixtos/data/DATOS_MIXTOS.xlsx
@@ -5,19 +5,19 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CN594\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Marti\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BB721C9-0522-4B2C-9FE3-FA1DD0B1EF96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B851F56-2D30-4367-AED9-E55BAEBBBB81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="21806" windowHeight="13886" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Proyectos" sheetId="1" r:id="rId1"/>
     <sheet name="Instrucciones" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Proyectos!$A$1:$P$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Proyectos!$A$1:$R$1</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="675" uniqueCount="365">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="734" uniqueCount="424">
   <si>
     <t>NO.</t>
   </si>
@@ -1132,6 +1132,183 @@
   </si>
   <si>
     <t>• PRIORI: escribe "P" si el proyecto es prioritario (aparece en el ranking del Resumen y su tarjeta se distingue) o "NoP" si no lo es.</t>
+  </si>
+  <si>
+    <t>name_BD</t>
+  </si>
+  <si>
+    <t>La Noria</t>
+  </si>
+  <si>
+    <t>PV Moquel Solar</t>
+  </si>
+  <si>
+    <t>PV Sandom Solar</t>
+  </si>
+  <si>
+    <t>Viento de Bella Unión</t>
+  </si>
+  <si>
+    <t>San Simón Solar</t>
+  </si>
+  <si>
+    <t>Solitario</t>
+  </si>
+  <si>
+    <t>Álvaro Obregón</t>
+  </si>
+  <si>
+    <t>Santa Gertrudis</t>
+  </si>
+  <si>
+    <t>El Guajillo</t>
+  </si>
+  <si>
+    <t>Tres Hermanos</t>
+  </si>
+  <si>
+    <t>Los Girasoles</t>
+  </si>
+  <si>
+    <t>Don Humberto</t>
+  </si>
+  <si>
+    <t>Haab Kiin</t>
+  </si>
+  <si>
+    <t>Planta Solar Cerro Colorado</t>
+  </si>
+  <si>
+    <t>CFV Quasara</t>
+  </si>
+  <si>
+    <t>Tikinmul</t>
+  </si>
+  <si>
+    <t>El Palmar</t>
+  </si>
+  <si>
+    <t>La Pasión</t>
+  </si>
+  <si>
+    <t>San Pedro Solar</t>
+  </si>
+  <si>
+    <t>Energía Limpia el Mezquite</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Energías Renovables De México Tres (Hecelchakan) </t>
+  </si>
+  <si>
+    <t>Energías Renovables Saas (Peto)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Energías Renovables Kiin (Tekax) </t>
+  </si>
+  <si>
+    <t>Energías Renovables de Tamaulipas (Altamira)</t>
+  </si>
+  <si>
+    <t>Dalia 3 (Castamay)</t>
+  </si>
+  <si>
+    <t>Fresnillo (PV Atocha)</t>
+  </si>
+  <si>
+    <t>Los Molinos</t>
+  </si>
+  <si>
+    <t>Montecristo</t>
+  </si>
+  <si>
+    <t>Sol de Sonora 70</t>
+  </si>
+  <si>
+    <t>Selka Power Plant 1</t>
+  </si>
+  <si>
+    <t>Concepción Mendizábal M. - Fase I</t>
+  </si>
+  <si>
+    <t>Concepción Mendizábal M. - Fase II</t>
+  </si>
+  <si>
+    <t>Concepción Mendizábal M. - Fase III</t>
+  </si>
+  <si>
+    <t>Global Solar 3 Campeche</t>
+  </si>
+  <si>
+    <t>CFV Las Garzas (**)</t>
+  </si>
+  <si>
+    <t>Cimarrón Solar (**)</t>
+  </si>
+  <si>
+    <t>Sunora (**)</t>
+  </si>
+  <si>
+    <t>La Poza Solar (**)</t>
+  </si>
+  <si>
+    <t>Sierra Madre (El Chorro) (*)</t>
+  </si>
+  <si>
+    <t>Delaro (*)</t>
+  </si>
+  <si>
+    <t>DI_LT</t>
+  </si>
+  <si>
+    <t>DI_P</t>
+  </si>
+  <si>
+    <t>ES_INT</t>
+  </si>
+  <si>
+    <t>A_MIA_P</t>
+  </si>
+  <si>
+    <t>A_MIA_LT</t>
+  </si>
+  <si>
+    <t>A_ETJ_LT</t>
+  </si>
+  <si>
+    <t>A_ETJ_P</t>
+  </si>
+  <si>
+    <t>S_MISSE_C</t>
+  </si>
+  <si>
+    <t>S_MISSE_LT</t>
+  </si>
+  <si>
+    <t>S_CONS</t>
+  </si>
+  <si>
+    <t>INAH_C</t>
+  </si>
+  <si>
+    <t>INAH_LT</t>
+  </si>
+  <si>
+    <t>PEMEX_C</t>
+  </si>
+  <si>
+    <t>PEMEX_LT</t>
+  </si>
+  <si>
+    <t>CONA_C</t>
+  </si>
+  <si>
+    <t>CONA_LT</t>
+  </si>
+  <si>
+    <t>AFAC_C</t>
+  </si>
+  <si>
+    <t>AFAC_LT</t>
   </si>
 </sst>
 </file>
@@ -1205,12 +1382,13 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1220,10 +1398,14 @@
     <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="3" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="3">
+  <cellStyles count="4">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 3" xfId="1" xr:uid="{BC78EB9C-0B95-49BA-A215-19B72E1CCE9C}"/>
+    <cellStyle name="Percent" xfId="3" builtinId="5"/>
     <cellStyle name="Porcentaje 2" xfId="2" xr:uid="{CA71FA13-44C4-4E1C-91BB-9480ABF23869}"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1524,28 +1706,32 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q42"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:BM42"/>
+  <sheetFormatPr defaultColWidth="9.15234375" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="4.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="47.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="22.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="33.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="25.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="37.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="21.7109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="23.28515625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="23.85546875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.28515625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="6.28515625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="7.5703125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="4.84375" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="47.84375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.53515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.69140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="33.69140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="25.15234375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="37.53515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21.69140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="23.3046875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="23.84375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17.3828125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.69140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.3046875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="6.3046875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="7.53515625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.84375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="14.3046875" customWidth="1"/>
+    <col min="22" max="26" width="12.4609375" customWidth="1"/>
+    <col min="27" max="27" width="11.84375" bestFit="1" customWidth="1"/>
+    <col min="28" max="36" width="12.4609375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:65" ht="28.3" x14ac:dyDescent="0.4">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -1597,8 +1783,94 @@
       <c r="Q1" s="6" t="s">
         <v>361</v>
       </c>
+      <c r="R1" s="6" t="s">
+        <v>365</v>
+      </c>
+      <c r="S1" s="6" t="s">
+        <v>407</v>
+      </c>
+      <c r="T1" s="6" t="s">
+        <v>406</v>
+      </c>
+      <c r="U1" s="6" t="s">
+        <v>408</v>
+      </c>
+      <c r="V1" s="6" t="s">
+        <v>409</v>
+      </c>
+      <c r="W1" s="6" t="s">
+        <v>410</v>
+      </c>
+      <c r="X1" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="Y1" s="6" t="s">
+        <v>411</v>
+      </c>
+      <c r="Z1" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="AA1" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="AB1" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="AC1" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="AD1" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="AE1" s="6" t="s">
+        <v>418</v>
+      </c>
+      <c r="AF1" s="6" t="s">
+        <v>419</v>
+      </c>
+      <c r="AG1" s="6" t="s">
+        <v>420</v>
+      </c>
+      <c r="AH1" s="6" t="s">
+        <v>421</v>
+      </c>
+      <c r="AI1" s="6" t="s">
+        <v>422</v>
+      </c>
+      <c r="AJ1" s="6" t="s">
+        <v>423</v>
+      </c>
+      <c r="AK1" s="8"/>
+      <c r="AL1" s="8"/>
+      <c r="AM1" s="8"/>
+      <c r="AN1" s="8"/>
+      <c r="AO1" s="8"/>
+      <c r="AP1" s="8"/>
+      <c r="AQ1" s="8"/>
+      <c r="AR1" s="8"/>
+      <c r="AS1" s="8"/>
+      <c r="AT1" s="8"/>
+      <c r="AU1" s="8"/>
+      <c r="AV1" s="8"/>
+      <c r="AW1" s="8"/>
+      <c r="AX1" s="8"/>
+      <c r="AY1" s="8"/>
+      <c r="AZ1" s="8"/>
+      <c r="BA1" s="8"/>
+      <c r="BB1" s="8"/>
+      <c r="BC1" s="8"/>
+      <c r="BD1" s="8"/>
+      <c r="BE1" s="8"/>
+      <c r="BF1" s="8"/>
+      <c r="BG1" s="8"/>
+      <c r="BH1" s="8"/>
+      <c r="BI1" s="8"/>
+      <c r="BJ1" s="8"/>
+      <c r="BK1" s="8"/>
+      <c r="BL1" s="8"/>
+      <c r="BM1" s="8"/>
     </row>
-    <row r="2" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:65" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -1650,8 +1922,94 @@
       <c r="Q2" s="1" t="s">
         <v>362</v>
       </c>
+      <c r="R2" s="7" t="s">
+        <v>370</v>
+      </c>
+      <c r="S2" s="9">
+        <v>1</v>
+      </c>
+      <c r="T2" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="U2" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="V2" s="9">
+        <v>1</v>
+      </c>
+      <c r="W2" s="9">
+        <v>1</v>
+      </c>
+      <c r="X2" s="9">
+        <v>1</v>
+      </c>
+      <c r="Y2" s="9">
+        <v>1</v>
+      </c>
+      <c r="Z2" s="9">
+        <v>1</v>
+      </c>
+      <c r="AA2" s="9">
+        <v>1</v>
+      </c>
+      <c r="AB2" s="9">
+        <v>1</v>
+      </c>
+      <c r="AC2" s="9">
+        <v>1</v>
+      </c>
+      <c r="AD2" s="9">
+        <v>1</v>
+      </c>
+      <c r="AE2" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AF2" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AG2" s="9">
+        <v>1</v>
+      </c>
+      <c r="AH2" s="9">
+        <v>1</v>
+      </c>
+      <c r="AI2" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AJ2" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AK2" s="8"/>
+      <c r="AL2" s="8"/>
+      <c r="AM2" s="8"/>
+      <c r="AN2" s="8"/>
+      <c r="AO2" s="8"/>
+      <c r="AP2" s="8"/>
+      <c r="AQ2" s="8"/>
+      <c r="AR2" s="8"/>
+      <c r="AS2" s="8"/>
+      <c r="AT2" s="8"/>
+      <c r="AU2" s="8"/>
+      <c r="AV2" s="8"/>
+      <c r="AW2" s="8"/>
+      <c r="AX2" s="8"/>
+      <c r="AY2" s="8"/>
+      <c r="AZ2" s="8"/>
+      <c r="BA2" s="8"/>
+      <c r="BB2" s="8"/>
+      <c r="BC2" s="8"/>
+      <c r="BD2" s="8"/>
+      <c r="BE2" s="8"/>
+      <c r="BF2" s="8"/>
+      <c r="BG2" s="8"/>
+      <c r="BH2" s="8"/>
+      <c r="BI2" s="8"/>
+      <c r="BJ2" s="8"/>
+      <c r="BK2" s="8"/>
+      <c r="BL2" s="8"/>
+      <c r="BM2" s="8"/>
     </row>
-    <row r="3" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:65" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -1703,8 +2061,94 @@
       <c r="Q3" s="1" t="s">
         <v>363</v>
       </c>
+      <c r="R3" s="7" t="s">
+        <v>366</v>
+      </c>
+      <c r="S3" s="9">
+        <v>1</v>
+      </c>
+      <c r="T3" s="9">
+        <v>1</v>
+      </c>
+      <c r="U3" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="V3" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="W3" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="X3" s="9">
+        <v>0.25</v>
+      </c>
+      <c r="Y3" s="9">
+        <v>0.25</v>
+      </c>
+      <c r="Z3" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="AA3" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="AB3" s="9">
+        <v>1</v>
+      </c>
+      <c r="AC3" s="9">
+        <v>0</v>
+      </c>
+      <c r="AD3" s="9">
+        <v>0</v>
+      </c>
+      <c r="AE3" s="9">
+        <v>0</v>
+      </c>
+      <c r="AF3" s="9">
+        <v>0</v>
+      </c>
+      <c r="AG3" s="9">
+        <v>0.25</v>
+      </c>
+      <c r="AH3" s="9">
+        <v>0</v>
+      </c>
+      <c r="AI3" s="9">
+        <v>0</v>
+      </c>
+      <c r="AJ3" s="9">
+        <v>0</v>
+      </c>
+      <c r="AK3" s="8"/>
+      <c r="AL3" s="8"/>
+      <c r="AM3" s="8"/>
+      <c r="AN3" s="8"/>
+      <c r="AO3" s="8"/>
+      <c r="AP3" s="8"/>
+      <c r="AQ3" s="8"/>
+      <c r="AR3" s="8"/>
+      <c r="AS3" s="8"/>
+      <c r="AT3" s="8"/>
+      <c r="AU3" s="8"/>
+      <c r="AV3" s="8"/>
+      <c r="AW3" s="8"/>
+      <c r="AX3" s="8"/>
+      <c r="AY3" s="8"/>
+      <c r="AZ3" s="8"/>
+      <c r="BA3" s="8"/>
+      <c r="BB3" s="8"/>
+      <c r="BC3" s="8"/>
+      <c r="BD3" s="8"/>
+      <c r="BE3" s="8"/>
+      <c r="BF3" s="8"/>
+      <c r="BG3" s="8"/>
+      <c r="BH3" s="8"/>
+      <c r="BI3" s="8"/>
+      <c r="BJ3" s="8"/>
+      <c r="BK3" s="8"/>
+      <c r="BL3" s="8"/>
+      <c r="BM3" s="8"/>
     </row>
-    <row r="4" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:65" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -1756,8 +2200,94 @@
       <c r="Q4" s="5" t="s">
         <v>363</v>
       </c>
+      <c r="R4" s="7" t="s">
+        <v>371</v>
+      </c>
+      <c r="S4" s="9">
+        <v>1</v>
+      </c>
+      <c r="T4" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="U4" s="9">
+        <v>1</v>
+      </c>
+      <c r="V4" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="W4" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="X4" s="9">
+        <v>0.25</v>
+      </c>
+      <c r="Y4" s="9">
+        <v>0.25</v>
+      </c>
+      <c r="Z4" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="AA4" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="AB4" s="9">
+        <v>1</v>
+      </c>
+      <c r="AC4" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="AD4" s="9">
+        <v>0</v>
+      </c>
+      <c r="AE4" s="9">
+        <v>0</v>
+      </c>
+      <c r="AF4" s="9">
+        <v>0</v>
+      </c>
+      <c r="AG4" s="9">
+        <v>0</v>
+      </c>
+      <c r="AH4" s="9">
+        <v>0</v>
+      </c>
+      <c r="AI4" s="9">
+        <v>0</v>
+      </c>
+      <c r="AJ4" s="9">
+        <v>0</v>
+      </c>
+      <c r="AK4" s="8"/>
+      <c r="AL4" s="8"/>
+      <c r="AM4" s="8"/>
+      <c r="AN4" s="8"/>
+      <c r="AO4" s="8"/>
+      <c r="AP4" s="8"/>
+      <c r="AQ4" s="8"/>
+      <c r="AR4" s="8"/>
+      <c r="AS4" s="8"/>
+      <c r="AT4" s="8"/>
+      <c r="AU4" s="8"/>
+      <c r="AV4" s="8"/>
+      <c r="AW4" s="8"/>
+      <c r="AX4" s="8"/>
+      <c r="AY4" s="8"/>
+      <c r="AZ4" s="8"/>
+      <c r="BA4" s="8"/>
+      <c r="BB4" s="8"/>
+      <c r="BC4" s="8"/>
+      <c r="BD4" s="8"/>
+      <c r="BE4" s="8"/>
+      <c r="BF4" s="8"/>
+      <c r="BG4" s="8"/>
+      <c r="BH4" s="8"/>
+      <c r="BI4" s="8"/>
+      <c r="BJ4" s="8"/>
+      <c r="BK4" s="8"/>
+      <c r="BL4" s="8"/>
+      <c r="BM4" s="8"/>
     </row>
-    <row r="5" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:65" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -1809,8 +2339,94 @@
       <c r="Q5" s="5" t="s">
         <v>362</v>
       </c>
+      <c r="R5" s="7" t="s">
+        <v>372</v>
+      </c>
+      <c r="S5" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="T5" s="9">
+        <v>0.8</v>
+      </c>
+      <c r="U5" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="V5" s="9">
+        <v>0.8</v>
+      </c>
+      <c r="W5" s="9">
+        <v>0.8</v>
+      </c>
+      <c r="X5" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="Y5" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="Z5" s="9">
+        <v>1</v>
+      </c>
+      <c r="AA5" s="9">
+        <v>1</v>
+      </c>
+      <c r="AB5" s="9">
+        <v>1</v>
+      </c>
+      <c r="AC5" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AD5" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AE5" s="9">
+        <v>1</v>
+      </c>
+      <c r="AF5" s="9">
+        <v>1</v>
+      </c>
+      <c r="AG5" s="9">
+        <v>1</v>
+      </c>
+      <c r="AH5" s="9">
+        <v>1</v>
+      </c>
+      <c r="AI5" s="9">
+        <v>1</v>
+      </c>
+      <c r="AJ5" s="9">
+        <v>1</v>
+      </c>
+      <c r="AK5" s="8"/>
+      <c r="AL5" s="8"/>
+      <c r="AM5" s="8"/>
+      <c r="AN5" s="8"/>
+      <c r="AO5" s="8"/>
+      <c r="AP5" s="8"/>
+      <c r="AQ5" s="8"/>
+      <c r="AR5" s="8"/>
+      <c r="AS5" s="8"/>
+      <c r="AT5" s="8"/>
+      <c r="AU5" s="8"/>
+      <c r="AV5" s="8"/>
+      <c r="AW5" s="8"/>
+      <c r="AX5" s="8"/>
+      <c r="AY5" s="8"/>
+      <c r="AZ5" s="8"/>
+      <c r="BA5" s="8"/>
+      <c r="BB5" s="8"/>
+      <c r="BC5" s="8"/>
+      <c r="BD5" s="8"/>
+      <c r="BE5" s="8"/>
+      <c r="BF5" s="8"/>
+      <c r="BG5" s="8"/>
+      <c r="BH5" s="8"/>
+      <c r="BI5" s="8"/>
+      <c r="BJ5" s="8"/>
+      <c r="BK5" s="8"/>
+      <c r="BL5" s="8"/>
+      <c r="BM5" s="8"/>
     </row>
-    <row r="6" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:65" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -1862,8 +2478,94 @@
       <c r="Q6" s="5" t="s">
         <v>362</v>
       </c>
+      <c r="R6" s="7" t="s">
+        <v>368</v>
+      </c>
+      <c r="S6" s="9">
+        <v>1</v>
+      </c>
+      <c r="T6" s="9">
+        <v>0</v>
+      </c>
+      <c r="U6" s="9">
+        <v>1</v>
+      </c>
+      <c r="V6" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="W6" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="X6" s="9">
+        <v>1</v>
+      </c>
+      <c r="Y6" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z6" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="AA6" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="AB6" s="9">
+        <v>0</v>
+      </c>
+      <c r="AC6" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="AD6" s="9">
+        <v>0</v>
+      </c>
+      <c r="AE6" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="AF6" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="AG6" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="AH6" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="AI6" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="AJ6" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="AK6" s="8"/>
+      <c r="AL6" s="8"/>
+      <c r="AM6" s="8"/>
+      <c r="AN6" s="8"/>
+      <c r="AO6" s="8"/>
+      <c r="AP6" s="8"/>
+      <c r="AQ6" s="8"/>
+      <c r="AR6" s="8"/>
+      <c r="AS6" s="8"/>
+      <c r="AT6" s="8"/>
+      <c r="AU6" s="8"/>
+      <c r="AV6" s="8"/>
+      <c r="AW6" s="8"/>
+      <c r="AX6" s="8"/>
+      <c r="AY6" s="8"/>
+      <c r="AZ6" s="8"/>
+      <c r="BA6" s="8"/>
+      <c r="BB6" s="8"/>
+      <c r="BC6" s="8"/>
+      <c r="BD6" s="8"/>
+      <c r="BE6" s="8"/>
+      <c r="BF6" s="8"/>
+      <c r="BG6" s="8"/>
+      <c r="BH6" s="8"/>
+      <c r="BI6" s="8"/>
+      <c r="BJ6" s="8"/>
+      <c r="BK6" s="8"/>
+      <c r="BL6" s="8"/>
+      <c r="BM6" s="8"/>
     </row>
-    <row r="7" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:65" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -1915,8 +2617,94 @@
       <c r="Q7" s="5" t="s">
         <v>363</v>
       </c>
+      <c r="R7" s="7" t="s">
+        <v>373</v>
+      </c>
+      <c r="S7" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="T7" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="U7" s="9">
+        <v>1</v>
+      </c>
+      <c r="V7" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="W7" s="9">
+        <v>0</v>
+      </c>
+      <c r="X7" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="Y7" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z7" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AA7" s="9">
+        <v>0</v>
+      </c>
+      <c r="AB7" s="9">
+        <v>1</v>
+      </c>
+      <c r="AC7" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AD7" s="9">
+        <v>0</v>
+      </c>
+      <c r="AE7" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AF7" s="9">
+        <v>0</v>
+      </c>
+      <c r="AG7" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AH7" s="9">
+        <v>0</v>
+      </c>
+      <c r="AI7" s="9">
+        <v>0</v>
+      </c>
+      <c r="AJ7" s="9">
+        <v>0</v>
+      </c>
+      <c r="AK7" s="8"/>
+      <c r="AL7" s="8"/>
+      <c r="AM7" s="8"/>
+      <c r="AN7" s="8"/>
+      <c r="AO7" s="8"/>
+      <c r="AP7" s="8"/>
+      <c r="AQ7" s="8"/>
+      <c r="AR7" s="8"/>
+      <c r="AS7" s="8"/>
+      <c r="AT7" s="8"/>
+      <c r="AU7" s="8"/>
+      <c r="AV7" s="8"/>
+      <c r="AW7" s="8"/>
+      <c r="AX7" s="8"/>
+      <c r="AY7" s="8"/>
+      <c r="AZ7" s="8"/>
+      <c r="BA7" s="8"/>
+      <c r="BB7" s="8"/>
+      <c r="BC7" s="8"/>
+      <c r="BD7" s="8"/>
+      <c r="BE7" s="8"/>
+      <c r="BF7" s="8"/>
+      <c r="BG7" s="8"/>
+      <c r="BH7" s="8"/>
+      <c r="BI7" s="8"/>
+      <c r="BJ7" s="8"/>
+      <c r="BK7" s="8"/>
+      <c r="BL7" s="8"/>
+      <c r="BM7" s="8"/>
     </row>
-    <row r="8" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:65" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -1968,8 +2756,94 @@
       <c r="Q8" s="5" t="s">
         <v>363</v>
       </c>
+      <c r="R8" s="7" t="s">
+        <v>374</v>
+      </c>
+      <c r="S8" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="T8" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="U8" s="9">
+        <v>1</v>
+      </c>
+      <c r="V8" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="W8" s="9">
+        <v>0</v>
+      </c>
+      <c r="X8" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="Y8" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z8" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AA8" s="9">
+        <v>0</v>
+      </c>
+      <c r="AB8" s="9">
+        <v>1</v>
+      </c>
+      <c r="AC8" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AD8" s="9">
+        <v>0</v>
+      </c>
+      <c r="AE8" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AF8" s="9">
+        <v>0</v>
+      </c>
+      <c r="AG8" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AH8" s="9">
+        <v>0</v>
+      </c>
+      <c r="AI8" s="9">
+        <v>0</v>
+      </c>
+      <c r="AJ8" s="9">
+        <v>0</v>
+      </c>
+      <c r="AK8" s="8"/>
+      <c r="AL8" s="8"/>
+      <c r="AM8" s="8"/>
+      <c r="AN8" s="8"/>
+      <c r="AO8" s="8"/>
+      <c r="AP8" s="8"/>
+      <c r="AQ8" s="8"/>
+      <c r="AR8" s="8"/>
+      <c r="AS8" s="8"/>
+      <c r="AT8" s="8"/>
+      <c r="AU8" s="8"/>
+      <c r="AV8" s="8"/>
+      <c r="AW8" s="8"/>
+      <c r="AX8" s="8"/>
+      <c r="AY8" s="8"/>
+      <c r="AZ8" s="8"/>
+      <c r="BA8" s="8"/>
+      <c r="BB8" s="8"/>
+      <c r="BC8" s="8"/>
+      <c r="BD8" s="8"/>
+      <c r="BE8" s="8"/>
+      <c r="BF8" s="8"/>
+      <c r="BG8" s="8"/>
+      <c r="BH8" s="8"/>
+      <c r="BI8" s="8"/>
+      <c r="BJ8" s="8"/>
+      <c r="BK8" s="8"/>
+      <c r="BL8" s="8"/>
+      <c r="BM8" s="8"/>
     </row>
-    <row r="9" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:65" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -2021,8 +2895,94 @@
       <c r="Q9" s="5" t="s">
         <v>363</v>
       </c>
+      <c r="R9" s="7" t="s">
+        <v>375</v>
+      </c>
+      <c r="S9" s="9">
+        <v>1</v>
+      </c>
+      <c r="T9" s="9">
+        <v>0</v>
+      </c>
+      <c r="U9" s="9">
+        <v>1</v>
+      </c>
+      <c r="V9" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="W9" s="9">
+        <v>0</v>
+      </c>
+      <c r="X9" s="9">
+        <v>1</v>
+      </c>
+      <c r="Y9" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z9" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="AA9" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="AB9" s="9">
+        <v>0</v>
+      </c>
+      <c r="AC9" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AD9" s="9">
+        <v>0</v>
+      </c>
+      <c r="AE9" s="9">
+        <v>1</v>
+      </c>
+      <c r="AF9" s="9">
+        <v>1</v>
+      </c>
+      <c r="AG9" s="9">
+        <v>0</v>
+      </c>
+      <c r="AH9" s="9">
+        <v>0</v>
+      </c>
+      <c r="AI9" s="9">
+        <v>0</v>
+      </c>
+      <c r="AJ9" s="9">
+        <v>0</v>
+      </c>
+      <c r="AK9" s="8"/>
+      <c r="AL9" s="8"/>
+      <c r="AM9" s="8"/>
+      <c r="AN9" s="8"/>
+      <c r="AO9" s="8"/>
+      <c r="AP9" s="8"/>
+      <c r="AQ9" s="8"/>
+      <c r="AR9" s="8"/>
+      <c r="AS9" s="8"/>
+      <c r="AT9" s="8"/>
+      <c r="AU9" s="8"/>
+      <c r="AV9" s="8"/>
+      <c r="AW9" s="8"/>
+      <c r="AX9" s="8"/>
+      <c r="AY9" s="8"/>
+      <c r="AZ9" s="8"/>
+      <c r="BA9" s="8"/>
+      <c r="BB9" s="8"/>
+      <c r="BC9" s="8"/>
+      <c r="BD9" s="8"/>
+      <c r="BE9" s="8"/>
+      <c r="BF9" s="8"/>
+      <c r="BG9" s="8"/>
+      <c r="BH9" s="8"/>
+      <c r="BI9" s="8"/>
+      <c r="BJ9" s="8"/>
+      <c r="BK9" s="8"/>
+      <c r="BL9" s="8"/>
+      <c r="BM9" s="8"/>
     </row>
-    <row r="10" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:65" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -2074,8 +3034,94 @@
       <c r="Q10" s="5" t="s">
         <v>363</v>
       </c>
+      <c r="R10" s="7" t="s">
+        <v>376</v>
+      </c>
+      <c r="S10" s="9">
+        <v>1</v>
+      </c>
+      <c r="T10" s="9">
+        <v>1</v>
+      </c>
+      <c r="U10" s="9">
+        <v>1</v>
+      </c>
+      <c r="V10" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="W10" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="X10" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="Y10" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="Z10" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="AA10" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="AB10" s="9">
+        <v>0</v>
+      </c>
+      <c r="AC10" s="9">
+        <v>0</v>
+      </c>
+      <c r="AD10" s="9">
+        <v>0</v>
+      </c>
+      <c r="AE10" s="9">
+        <v>1</v>
+      </c>
+      <c r="AF10" s="9">
+        <v>1</v>
+      </c>
+      <c r="AG10" s="9">
+        <v>0</v>
+      </c>
+      <c r="AH10" s="9">
+        <v>0</v>
+      </c>
+      <c r="AI10" s="9">
+        <v>0</v>
+      </c>
+      <c r="AJ10" s="9">
+        <v>0</v>
+      </c>
+      <c r="AK10" s="8"/>
+      <c r="AL10" s="8"/>
+      <c r="AM10" s="8"/>
+      <c r="AN10" s="8"/>
+      <c r="AO10" s="8"/>
+      <c r="AP10" s="8"/>
+      <c r="AQ10" s="8"/>
+      <c r="AR10" s="8"/>
+      <c r="AS10" s="8"/>
+      <c r="AT10" s="8"/>
+      <c r="AU10" s="8"/>
+      <c r="AV10" s="8"/>
+      <c r="AW10" s="8"/>
+      <c r="AX10" s="8"/>
+      <c r="AY10" s="8"/>
+      <c r="AZ10" s="8"/>
+      <c r="BA10" s="8"/>
+      <c r="BB10" s="8"/>
+      <c r="BC10" s="8"/>
+      <c r="BD10" s="8"/>
+      <c r="BE10" s="8"/>
+      <c r="BF10" s="8"/>
+      <c r="BG10" s="8"/>
+      <c r="BH10" s="8"/>
+      <c r="BI10" s="8"/>
+      <c r="BJ10" s="8"/>
+      <c r="BK10" s="8"/>
+      <c r="BL10" s="8"/>
+      <c r="BM10" s="8"/>
     </row>
-    <row r="11" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:65" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -2127,8 +3173,94 @@
       <c r="Q11" s="5" t="s">
         <v>362</v>
       </c>
+      <c r="R11" s="7" t="s">
+        <v>377</v>
+      </c>
+      <c r="S11" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="T11" s="9">
+        <v>0</v>
+      </c>
+      <c r="U11" s="9">
+        <v>1</v>
+      </c>
+      <c r="V11" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="W11" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="X11" s="9">
+        <v>1</v>
+      </c>
+      <c r="Y11" s="9">
+        <v>1</v>
+      </c>
+      <c r="Z11" s="9">
+        <v>0.8</v>
+      </c>
+      <c r="AA11" s="9">
+        <v>0.8</v>
+      </c>
+      <c r="AB11" s="9">
+        <v>1</v>
+      </c>
+      <c r="AC11" s="9">
+        <v>1</v>
+      </c>
+      <c r="AD11" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AE11" s="9">
+        <v>1</v>
+      </c>
+      <c r="AF11" s="9">
+        <v>1</v>
+      </c>
+      <c r="AG11" s="9">
+        <v>0</v>
+      </c>
+      <c r="AH11" s="9">
+        <v>0</v>
+      </c>
+      <c r="AI11" s="9">
+        <v>0</v>
+      </c>
+      <c r="AJ11" s="9">
+        <v>0</v>
+      </c>
+      <c r="AK11" s="8"/>
+      <c r="AL11" s="8"/>
+      <c r="AM11" s="8"/>
+      <c r="AN11" s="8"/>
+      <c r="AO11" s="8"/>
+      <c r="AP11" s="8"/>
+      <c r="AQ11" s="8"/>
+      <c r="AR11" s="8"/>
+      <c r="AS11" s="8"/>
+      <c r="AT11" s="8"/>
+      <c r="AU11" s="8"/>
+      <c r="AV11" s="8"/>
+      <c r="AW11" s="8"/>
+      <c r="AX11" s="8"/>
+      <c r="AY11" s="8"/>
+      <c r="AZ11" s="8"/>
+      <c r="BA11" s="8"/>
+      <c r="BB11" s="8"/>
+      <c r="BC11" s="8"/>
+      <c r="BD11" s="8"/>
+      <c r="BE11" s="8"/>
+      <c r="BF11" s="8"/>
+      <c r="BG11" s="8"/>
+      <c r="BH11" s="8"/>
+      <c r="BI11" s="8"/>
+      <c r="BJ11" s="8"/>
+      <c r="BK11" s="8"/>
+      <c r="BL11" s="8"/>
+      <c r="BM11" s="8"/>
     </row>
-    <row r="12" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:65" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -2180,8 +3312,94 @@
       <c r="Q12" s="5" t="s">
         <v>362</v>
       </c>
+      <c r="R12" s="7" t="s">
+        <v>378</v>
+      </c>
+      <c r="S12" s="9">
+        <v>1</v>
+      </c>
+      <c r="T12" s="9">
+        <v>0.75</v>
+      </c>
+      <c r="U12" s="9">
+        <v>1</v>
+      </c>
+      <c r="V12" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="W12" s="9">
+        <v>0.8</v>
+      </c>
+      <c r="X12" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="Y12" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="Z12" s="9">
+        <v>0.8</v>
+      </c>
+      <c r="AA12" s="9">
+        <v>0.8</v>
+      </c>
+      <c r="AB12" s="9">
+        <v>0</v>
+      </c>
+      <c r="AC12" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AD12" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AE12" s="9">
+        <v>1</v>
+      </c>
+      <c r="AF12" s="9">
+        <v>1</v>
+      </c>
+      <c r="AG12" s="9">
+        <v>1</v>
+      </c>
+      <c r="AH12" s="9">
+        <v>1</v>
+      </c>
+      <c r="AI12" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AJ12" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AK12" s="8"/>
+      <c r="AL12" s="8"/>
+      <c r="AM12" s="8"/>
+      <c r="AN12" s="8"/>
+      <c r="AO12" s="8"/>
+      <c r="AP12" s="8"/>
+      <c r="AQ12" s="8"/>
+      <c r="AR12" s="8"/>
+      <c r="AS12" s="8"/>
+      <c r="AT12" s="8"/>
+      <c r="AU12" s="8"/>
+      <c r="AV12" s="8"/>
+      <c r="AW12" s="8"/>
+      <c r="AX12" s="8"/>
+      <c r="AY12" s="8"/>
+      <c r="AZ12" s="8"/>
+      <c r="BA12" s="8"/>
+      <c r="BB12" s="8"/>
+      <c r="BC12" s="8"/>
+      <c r="BD12" s="8"/>
+      <c r="BE12" s="8"/>
+      <c r="BF12" s="8"/>
+      <c r="BG12" s="8"/>
+      <c r="BH12" s="8"/>
+      <c r="BI12" s="8"/>
+      <c r="BJ12" s="8"/>
+      <c r="BK12" s="8"/>
+      <c r="BL12" s="8"/>
+      <c r="BM12" s="8"/>
     </row>
-    <row r="13" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:65" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -2233,8 +3451,94 @@
       <c r="Q13" s="5" t="s">
         <v>363</v>
       </c>
+      <c r="R13" s="7" t="s">
+        <v>379</v>
+      </c>
+      <c r="S13" s="9">
+        <v>1</v>
+      </c>
+      <c r="T13" s="9">
+        <v>0.75</v>
+      </c>
+      <c r="U13" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="V13" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="W13" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="X13" s="9">
+        <v>1</v>
+      </c>
+      <c r="Y13" s="9">
+        <v>0.25</v>
+      </c>
+      <c r="Z13" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="AA13" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="AB13" s="9">
+        <v>0</v>
+      </c>
+      <c r="AC13" s="9">
+        <v>0.8</v>
+      </c>
+      <c r="AD13" s="9">
+        <v>0</v>
+      </c>
+      <c r="AE13" s="9">
+        <v>0.8</v>
+      </c>
+      <c r="AF13" s="9">
+        <v>0.8</v>
+      </c>
+      <c r="AG13" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AH13" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AI13" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AJ13" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AK13" s="8"/>
+      <c r="AL13" s="8"/>
+      <c r="AM13" s="8"/>
+      <c r="AN13" s="8"/>
+      <c r="AO13" s="8"/>
+      <c r="AP13" s="8"/>
+      <c r="AQ13" s="8"/>
+      <c r="AR13" s="8"/>
+      <c r="AS13" s="8"/>
+      <c r="AT13" s="8"/>
+      <c r="AU13" s="8"/>
+      <c r="AV13" s="8"/>
+      <c r="AW13" s="8"/>
+      <c r="AX13" s="8"/>
+      <c r="AY13" s="8"/>
+      <c r="AZ13" s="8"/>
+      <c r="BA13" s="8"/>
+      <c r="BB13" s="8"/>
+      <c r="BC13" s="8"/>
+      <c r="BD13" s="8"/>
+      <c r="BE13" s="8"/>
+      <c r="BF13" s="8"/>
+      <c r="BG13" s="8"/>
+      <c r="BH13" s="8"/>
+      <c r="BI13" s="8"/>
+      <c r="BJ13" s="8"/>
+      <c r="BK13" s="8"/>
+      <c r="BL13" s="8"/>
+      <c r="BM13" s="8"/>
     </row>
-    <row r="14" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:65" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A14" s="1">
         <v>13</v>
       </c>
@@ -2286,8 +3590,94 @@
       <c r="Q14" s="5" t="s">
         <v>363</v>
       </c>
+      <c r="R14" s="7" t="s">
+        <v>380</v>
+      </c>
+      <c r="S14" s="9">
+        <v>0.8</v>
+      </c>
+      <c r="T14" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="U14" s="9">
+        <v>1</v>
+      </c>
+      <c r="V14" s="9">
+        <v>0</v>
+      </c>
+      <c r="W14" s="9">
+        <v>0</v>
+      </c>
+      <c r="X14" s="9">
+        <v>0</v>
+      </c>
+      <c r="Y14" s="9">
+        <v>1</v>
+      </c>
+      <c r="Z14" s="9">
+        <v>0</v>
+      </c>
+      <c r="AA14" s="9">
+        <v>0</v>
+      </c>
+      <c r="AB14" s="9">
+        <v>0</v>
+      </c>
+      <c r="AC14" s="9">
+        <v>0</v>
+      </c>
+      <c r="AD14" s="9">
+        <v>0</v>
+      </c>
+      <c r="AE14" s="9">
+        <v>0</v>
+      </c>
+      <c r="AF14" s="9">
+        <v>0</v>
+      </c>
+      <c r="AG14" s="9">
+        <v>0</v>
+      </c>
+      <c r="AH14" s="9">
+        <v>0</v>
+      </c>
+      <c r="AI14" s="9">
+        <v>0</v>
+      </c>
+      <c r="AJ14" s="9">
+        <v>0</v>
+      </c>
+      <c r="AK14" s="8"/>
+      <c r="AL14" s="8"/>
+      <c r="AM14" s="8"/>
+      <c r="AN14" s="8"/>
+      <c r="AO14" s="8"/>
+      <c r="AP14" s="8"/>
+      <c r="AQ14" s="8"/>
+      <c r="AR14" s="8"/>
+      <c r="AS14" s="8"/>
+      <c r="AT14" s="8"/>
+      <c r="AU14" s="8"/>
+      <c r="AV14" s="8"/>
+      <c r="AW14" s="8"/>
+      <c r="AX14" s="8"/>
+      <c r="AY14" s="8"/>
+      <c r="AZ14" s="8"/>
+      <c r="BA14" s="8"/>
+      <c r="BB14" s="8"/>
+      <c r="BC14" s="8"/>
+      <c r="BD14" s="8"/>
+      <c r="BE14" s="8"/>
+      <c r="BF14" s="8"/>
+      <c r="BG14" s="8"/>
+      <c r="BH14" s="8"/>
+      <c r="BI14" s="8"/>
+      <c r="BJ14" s="8"/>
+      <c r="BK14" s="8"/>
+      <c r="BL14" s="8"/>
+      <c r="BM14" s="8"/>
     </row>
-    <row r="15" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:65" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A15" s="1">
         <v>14</v>
       </c>
@@ -2339,8 +3729,94 @@
       <c r="Q15" s="5" t="s">
         <v>363</v>
       </c>
+      <c r="R15" s="7" t="s">
+        <v>381</v>
+      </c>
+      <c r="S15" s="9">
+        <v>1</v>
+      </c>
+      <c r="T15" s="9">
+        <v>0.8</v>
+      </c>
+      <c r="U15" s="9">
+        <v>0.8</v>
+      </c>
+      <c r="V15" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="W15" s="9">
+        <v>0</v>
+      </c>
+      <c r="X15" s="9">
+        <v>0</v>
+      </c>
+      <c r="Y15" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z15" s="9">
+        <v>0</v>
+      </c>
+      <c r="AA15" s="9">
+        <v>0</v>
+      </c>
+      <c r="AB15" s="9">
+        <v>0</v>
+      </c>
+      <c r="AC15" s="9">
+        <v>0</v>
+      </c>
+      <c r="AD15" s="9">
+        <v>0</v>
+      </c>
+      <c r="AE15" s="9">
+        <v>0</v>
+      </c>
+      <c r="AF15" s="9">
+        <v>0</v>
+      </c>
+      <c r="AG15" s="9">
+        <v>0</v>
+      </c>
+      <c r="AH15" s="9">
+        <v>0</v>
+      </c>
+      <c r="AI15" s="9">
+        <v>0</v>
+      </c>
+      <c r="AJ15" s="9">
+        <v>0</v>
+      </c>
+      <c r="AK15" s="8"/>
+      <c r="AL15" s="8"/>
+      <c r="AM15" s="8"/>
+      <c r="AN15" s="8"/>
+      <c r="AO15" s="8"/>
+      <c r="AP15" s="8"/>
+      <c r="AQ15" s="8"/>
+      <c r="AR15" s="8"/>
+      <c r="AS15" s="8"/>
+      <c r="AT15" s="8"/>
+      <c r="AU15" s="8"/>
+      <c r="AV15" s="8"/>
+      <c r="AW15" s="8"/>
+      <c r="AX15" s="8"/>
+      <c r="AY15" s="8"/>
+      <c r="AZ15" s="8"/>
+      <c r="BA15" s="8"/>
+      <c r="BB15" s="8"/>
+      <c r="BC15" s="8"/>
+      <c r="BD15" s="8"/>
+      <c r="BE15" s="8"/>
+      <c r="BF15" s="8"/>
+      <c r="BG15" s="8"/>
+      <c r="BH15" s="8"/>
+      <c r="BI15" s="8"/>
+      <c r="BJ15" s="8"/>
+      <c r="BK15" s="8"/>
+      <c r="BL15" s="8"/>
+      <c r="BM15" s="8"/>
     </row>
-    <row r="16" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:65" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A16" s="1">
         <v>15</v>
       </c>
@@ -2392,8 +3868,94 @@
       <c r="Q16" s="5" t="s">
         <v>363</v>
       </c>
+      <c r="R16" s="7" t="s">
+        <v>382</v>
+      </c>
+      <c r="S16" s="9">
+        <v>1</v>
+      </c>
+      <c r="T16" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="U16" s="9">
+        <v>0.8</v>
+      </c>
+      <c r="V16" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="W16" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="X16" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="Y16" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="Z16" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AA16" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AB16" s="9">
+        <v>1</v>
+      </c>
+      <c r="AC16" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AD16" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AE16" s="9">
+        <v>0</v>
+      </c>
+      <c r="AF16" s="9">
+        <v>0</v>
+      </c>
+      <c r="AG16" s="9">
+        <v>0</v>
+      </c>
+      <c r="AH16" s="9">
+        <v>0</v>
+      </c>
+      <c r="AI16" s="9">
+        <v>0</v>
+      </c>
+      <c r="AJ16" s="9">
+        <v>0</v>
+      </c>
+      <c r="AK16" s="8"/>
+      <c r="AL16" s="8"/>
+      <c r="AM16" s="8"/>
+      <c r="AN16" s="8"/>
+      <c r="AO16" s="8"/>
+      <c r="AP16" s="8"/>
+      <c r="AQ16" s="8"/>
+      <c r="AR16" s="8"/>
+      <c r="AS16" s="8"/>
+      <c r="AT16" s="8"/>
+      <c r="AU16" s="8"/>
+      <c r="AV16" s="8"/>
+      <c r="AW16" s="8"/>
+      <c r="AX16" s="8"/>
+      <c r="AY16" s="8"/>
+      <c r="AZ16" s="8"/>
+      <c r="BA16" s="8"/>
+      <c r="BB16" s="8"/>
+      <c r="BC16" s="8"/>
+      <c r="BD16" s="8"/>
+      <c r="BE16" s="8"/>
+      <c r="BF16" s="8"/>
+      <c r="BG16" s="8"/>
+      <c r="BH16" s="8"/>
+      <c r="BI16" s="8"/>
+      <c r="BJ16" s="8"/>
+      <c r="BK16" s="8"/>
+      <c r="BL16" s="8"/>
+      <c r="BM16" s="8"/>
     </row>
-    <row r="17" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:65" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A17" s="1">
         <v>16</v>
       </c>
@@ -2445,8 +4007,94 @@
       <c r="Q17" s="5" t="s">
         <v>363</v>
       </c>
+      <c r="R17" s="7" t="s">
+        <v>383</v>
+      </c>
+      <c r="S17" s="9">
+        <v>1</v>
+      </c>
+      <c r="T17" s="9">
+        <v>0.8</v>
+      </c>
+      <c r="U17" s="9">
+        <v>1</v>
+      </c>
+      <c r="V17" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="W17" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="X17" s="9">
+        <v>0.4</v>
+      </c>
+      <c r="Y17" s="9">
+        <v>0.4</v>
+      </c>
+      <c r="Z17" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AA17" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AB17" s="9">
+        <v>1</v>
+      </c>
+      <c r="AC17" s="9">
+        <v>0</v>
+      </c>
+      <c r="AD17" s="9">
+        <v>0</v>
+      </c>
+      <c r="AE17" s="9">
+        <v>0</v>
+      </c>
+      <c r="AF17" s="9">
+        <v>0</v>
+      </c>
+      <c r="AG17" s="9">
+        <v>0</v>
+      </c>
+      <c r="AH17" s="9">
+        <v>0</v>
+      </c>
+      <c r="AI17" s="9">
+        <v>0</v>
+      </c>
+      <c r="AJ17" s="9">
+        <v>0</v>
+      </c>
+      <c r="AK17" s="8"/>
+      <c r="AL17" s="8"/>
+      <c r="AM17" s="8"/>
+      <c r="AN17" s="8"/>
+      <c r="AO17" s="8"/>
+      <c r="AP17" s="8"/>
+      <c r="AQ17" s="8"/>
+      <c r="AR17" s="8"/>
+      <c r="AS17" s="8"/>
+      <c r="AT17" s="8"/>
+      <c r="AU17" s="8"/>
+      <c r="AV17" s="8"/>
+      <c r="AW17" s="8"/>
+      <c r="AX17" s="8"/>
+      <c r="AY17" s="8"/>
+      <c r="AZ17" s="8"/>
+      <c r="BA17" s="8"/>
+      <c r="BB17" s="8"/>
+      <c r="BC17" s="8"/>
+      <c r="BD17" s="8"/>
+      <c r="BE17" s="8"/>
+      <c r="BF17" s="8"/>
+      <c r="BG17" s="8"/>
+      <c r="BH17" s="8"/>
+      <c r="BI17" s="8"/>
+      <c r="BJ17" s="8"/>
+      <c r="BK17" s="8"/>
+      <c r="BL17" s="8"/>
+      <c r="BM17" s="8"/>
     </row>
-    <row r="18" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:65" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A18" s="1">
         <v>17</v>
       </c>
@@ -2498,8 +4146,94 @@
       <c r="Q18" s="5" t="s">
         <v>362</v>
       </c>
+      <c r="R18" s="7" t="s">
+        <v>384</v>
+      </c>
+      <c r="S18" s="9">
+        <v>0.95</v>
+      </c>
+      <c r="T18" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="U18" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="V18" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="W18" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="X18" s="9">
+        <v>1</v>
+      </c>
+      <c r="Y18" s="9">
+        <v>1</v>
+      </c>
+      <c r="Z18" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="AA18" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="AB18" s="9">
+        <v>1</v>
+      </c>
+      <c r="AC18" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="AD18" s="9">
+        <v>0.8</v>
+      </c>
+      <c r="AE18" s="9">
+        <v>1</v>
+      </c>
+      <c r="AF18" s="9">
+        <v>1</v>
+      </c>
+      <c r="AG18" s="9">
+        <v>0.8</v>
+      </c>
+      <c r="AH18" s="9">
+        <v>0.8</v>
+      </c>
+      <c r="AI18" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AJ18" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AK18" s="8"/>
+      <c r="AL18" s="8"/>
+      <c r="AM18" s="8"/>
+      <c r="AN18" s="8"/>
+      <c r="AO18" s="8"/>
+      <c r="AP18" s="8"/>
+      <c r="AQ18" s="8"/>
+      <c r="AR18" s="8"/>
+      <c r="AS18" s="8"/>
+      <c r="AT18" s="8"/>
+      <c r="AU18" s="8"/>
+      <c r="AV18" s="8"/>
+      <c r="AW18" s="8"/>
+      <c r="AX18" s="8"/>
+      <c r="AY18" s="8"/>
+      <c r="AZ18" s="8"/>
+      <c r="BA18" s="8"/>
+      <c r="BB18" s="8"/>
+      <c r="BC18" s="8"/>
+      <c r="BD18" s="8"/>
+      <c r="BE18" s="8"/>
+      <c r="BF18" s="8"/>
+      <c r="BG18" s="8"/>
+      <c r="BH18" s="8"/>
+      <c r="BI18" s="8"/>
+      <c r="BJ18" s="8"/>
+      <c r="BK18" s="8"/>
+      <c r="BL18" s="8"/>
+      <c r="BM18" s="8"/>
     </row>
-    <row r="19" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:65" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A19" s="1">
         <v>18</v>
       </c>
@@ -2551,8 +4285,94 @@
       <c r="Q19" s="5" t="s">
         <v>363</v>
       </c>
+      <c r="R19" s="7" t="s">
+        <v>385</v>
+      </c>
+      <c r="S19" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="T19" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="U19" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="V19" s="9">
+        <v>0.8</v>
+      </c>
+      <c r="W19" s="9">
+        <v>0.7</v>
+      </c>
+      <c r="X19" s="9">
+        <v>0.6</v>
+      </c>
+      <c r="Y19" s="9">
+        <v>0.6</v>
+      </c>
+      <c r="Z19" s="9">
+        <v>0.8</v>
+      </c>
+      <c r="AA19" s="9">
+        <v>0.8</v>
+      </c>
+      <c r="AB19" s="9">
+        <v>1</v>
+      </c>
+      <c r="AC19" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AD19" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AE19" s="9">
+        <v>0</v>
+      </c>
+      <c r="AF19" s="9">
+        <v>0</v>
+      </c>
+      <c r="AG19" s="9">
+        <v>0</v>
+      </c>
+      <c r="AH19" s="9">
+        <v>0</v>
+      </c>
+      <c r="AI19" s="9">
+        <v>0</v>
+      </c>
+      <c r="AJ19" s="9">
+        <v>0</v>
+      </c>
+      <c r="AK19" s="8"/>
+      <c r="AL19" s="8"/>
+      <c r="AM19" s="8"/>
+      <c r="AN19" s="8"/>
+      <c r="AO19" s="8"/>
+      <c r="AP19" s="8"/>
+      <c r="AQ19" s="8"/>
+      <c r="AR19" s="8"/>
+      <c r="AS19" s="8"/>
+      <c r="AT19" s="8"/>
+      <c r="AU19" s="8"/>
+      <c r="AV19" s="8"/>
+      <c r="AW19" s="8"/>
+      <c r="AX19" s="8"/>
+      <c r="AY19" s="8"/>
+      <c r="AZ19" s="8"/>
+      <c r="BA19" s="8"/>
+      <c r="BB19" s="8"/>
+      <c r="BC19" s="8"/>
+      <c r="BD19" s="8"/>
+      <c r="BE19" s="8"/>
+      <c r="BF19" s="8"/>
+      <c r="BG19" s="8"/>
+      <c r="BH19" s="8"/>
+      <c r="BI19" s="8"/>
+      <c r="BJ19" s="8"/>
+      <c r="BK19" s="8"/>
+      <c r="BL19" s="8"/>
+      <c r="BM19" s="8"/>
     </row>
-    <row r="20" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:65" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A20" s="1">
         <v>19</v>
       </c>
@@ -2604,8 +4424,94 @@
       <c r="Q20" s="5" t="s">
         <v>363</v>
       </c>
+      <c r="R20" s="7" t="s">
+        <v>386</v>
+      </c>
+      <c r="S20" s="9">
+        <v>1</v>
+      </c>
+      <c r="T20" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="U20" s="9">
+        <v>1</v>
+      </c>
+      <c r="V20" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="W20" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="X20" s="9">
+        <v>1</v>
+      </c>
+      <c r="Y20" s="9">
+        <v>1</v>
+      </c>
+      <c r="Z20" s="9">
+        <v>0.8</v>
+      </c>
+      <c r="AA20" s="9">
+        <v>0.8</v>
+      </c>
+      <c r="AB20" s="9">
+        <v>0</v>
+      </c>
+      <c r="AC20" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AD20" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AE20" s="9">
+        <v>1</v>
+      </c>
+      <c r="AF20" s="9">
+        <v>1</v>
+      </c>
+      <c r="AG20" s="9">
+        <v>1</v>
+      </c>
+      <c r="AH20" s="9">
+        <v>1</v>
+      </c>
+      <c r="AI20" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AJ20" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AK20" s="8"/>
+      <c r="AL20" s="8"/>
+      <c r="AM20" s="8"/>
+      <c r="AN20" s="8"/>
+      <c r="AO20" s="8"/>
+      <c r="AP20" s="8"/>
+      <c r="AQ20" s="8"/>
+      <c r="AR20" s="8"/>
+      <c r="AS20" s="8"/>
+      <c r="AT20" s="8"/>
+      <c r="AU20" s="8"/>
+      <c r="AV20" s="8"/>
+      <c r="AW20" s="8"/>
+      <c r="AX20" s="8"/>
+      <c r="AY20" s="8"/>
+      <c r="AZ20" s="8"/>
+      <c r="BA20" s="8"/>
+      <c r="BB20" s="8"/>
+      <c r="BC20" s="8"/>
+      <c r="BD20" s="8"/>
+      <c r="BE20" s="8"/>
+      <c r="BF20" s="8"/>
+      <c r="BG20" s="8"/>
+      <c r="BH20" s="8"/>
+      <c r="BI20" s="8"/>
+      <c r="BJ20" s="8"/>
+      <c r="BK20" s="8"/>
+      <c r="BL20" s="8"/>
+      <c r="BM20" s="8"/>
     </row>
-    <row r="21" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:65" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A21" s="1">
         <v>20</v>
       </c>
@@ -2657,8 +4563,94 @@
       <c r="Q21" s="5" t="s">
         <v>363</v>
       </c>
+      <c r="R21" s="7" t="s">
+        <v>387</v>
+      </c>
+      <c r="S21" s="9">
+        <v>1</v>
+      </c>
+      <c r="T21" s="9">
+        <v>0</v>
+      </c>
+      <c r="U21" s="9">
+        <v>1</v>
+      </c>
+      <c r="V21" s="9">
+        <v>0.8</v>
+      </c>
+      <c r="W21" s="9">
+        <v>0.8</v>
+      </c>
+      <c r="X21" s="9">
+        <v>0</v>
+      </c>
+      <c r="Y21" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z21" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="AA21" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="AB21" s="9">
+        <v>0</v>
+      </c>
+      <c r="AC21" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AD21" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AE21" s="9">
+        <v>1</v>
+      </c>
+      <c r="AF21" s="9">
+        <v>1</v>
+      </c>
+      <c r="AG21" s="9">
+        <v>1</v>
+      </c>
+      <c r="AH21" s="9">
+        <v>1</v>
+      </c>
+      <c r="AI21" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AJ21" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AK21" s="8"/>
+      <c r="AL21" s="8"/>
+      <c r="AM21" s="8"/>
+      <c r="AN21" s="8"/>
+      <c r="AO21" s="8"/>
+      <c r="AP21" s="8"/>
+      <c r="AQ21" s="8"/>
+      <c r="AR21" s="8"/>
+      <c r="AS21" s="8"/>
+      <c r="AT21" s="8"/>
+      <c r="AU21" s="8"/>
+      <c r="AV21" s="8"/>
+      <c r="AW21" s="8"/>
+      <c r="AX21" s="8"/>
+      <c r="AY21" s="8"/>
+      <c r="AZ21" s="8"/>
+      <c r="BA21" s="8"/>
+      <c r="BB21" s="8"/>
+      <c r="BC21" s="8"/>
+      <c r="BD21" s="8"/>
+      <c r="BE21" s="8"/>
+      <c r="BF21" s="8"/>
+      <c r="BG21" s="8"/>
+      <c r="BH21" s="8"/>
+      <c r="BI21" s="8"/>
+      <c r="BJ21" s="8"/>
+      <c r="BK21" s="8"/>
+      <c r="BL21" s="8"/>
+      <c r="BM21" s="8"/>
     </row>
-    <row r="22" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:65" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A22" s="1">
         <v>21</v>
       </c>
@@ -2710,8 +4702,94 @@
       <c r="Q22" s="5" t="s">
         <v>363</v>
       </c>
+      <c r="R22" s="7" t="s">
+        <v>388</v>
+      </c>
+      <c r="S22" s="9">
+        <v>1</v>
+      </c>
+      <c r="T22" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="U22" s="9">
+        <v>1</v>
+      </c>
+      <c r="V22" s="9">
+        <v>0.8</v>
+      </c>
+      <c r="W22" s="9">
+        <v>0.8</v>
+      </c>
+      <c r="X22" s="9">
+        <v>0</v>
+      </c>
+      <c r="Y22" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z22" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="AA22" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="AB22" s="9">
+        <v>0</v>
+      </c>
+      <c r="AC22" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AD22" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AE22" s="9">
+        <v>1</v>
+      </c>
+      <c r="AF22" s="9">
+        <v>1</v>
+      </c>
+      <c r="AG22" s="9">
+        <v>1</v>
+      </c>
+      <c r="AH22" s="9">
+        <v>1</v>
+      </c>
+      <c r="AI22" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AJ22" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AK22" s="8"/>
+      <c r="AL22" s="8"/>
+      <c r="AM22" s="8"/>
+      <c r="AN22" s="8"/>
+      <c r="AO22" s="8"/>
+      <c r="AP22" s="8"/>
+      <c r="AQ22" s="8"/>
+      <c r="AR22" s="8"/>
+      <c r="AS22" s="8"/>
+      <c r="AT22" s="8"/>
+      <c r="AU22" s="8"/>
+      <c r="AV22" s="8"/>
+      <c r="AW22" s="8"/>
+      <c r="AX22" s="8"/>
+      <c r="AY22" s="8"/>
+      <c r="AZ22" s="8"/>
+      <c r="BA22" s="8"/>
+      <c r="BB22" s="8"/>
+      <c r="BC22" s="8"/>
+      <c r="BD22" s="8"/>
+      <c r="BE22" s="8"/>
+      <c r="BF22" s="8"/>
+      <c r="BG22" s="8"/>
+      <c r="BH22" s="8"/>
+      <c r="BI22" s="8"/>
+      <c r="BJ22" s="8"/>
+      <c r="BK22" s="8"/>
+      <c r="BL22" s="8"/>
+      <c r="BM22" s="8"/>
     </row>
-    <row r="23" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:65" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A23" s="1">
         <v>22</v>
       </c>
@@ -2763,8 +4841,94 @@
       <c r="Q23" s="5" t="s">
         <v>362</v>
       </c>
+      <c r="R23" s="7" t="s">
+        <v>389</v>
+      </c>
+      <c r="S23" s="9">
+        <v>1</v>
+      </c>
+      <c r="T23" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="U23" s="9">
+        <v>1</v>
+      </c>
+      <c r="V23" s="9">
+        <v>0.8</v>
+      </c>
+      <c r="W23" s="9">
+        <v>0.8</v>
+      </c>
+      <c r="X23" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="Y23" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="Z23" s="9">
+        <v>1</v>
+      </c>
+      <c r="AA23" s="9">
+        <v>1</v>
+      </c>
+      <c r="AB23" s="9">
+        <v>1</v>
+      </c>
+      <c r="AC23" s="9">
+        <v>1</v>
+      </c>
+      <c r="AD23" s="9">
+        <v>1</v>
+      </c>
+      <c r="AE23" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AF23" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AG23" s="9">
+        <v>1</v>
+      </c>
+      <c r="AH23" s="9">
+        <v>1</v>
+      </c>
+      <c r="AI23" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AJ23" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AK23" s="8"/>
+      <c r="AL23" s="8"/>
+      <c r="AM23" s="8"/>
+      <c r="AN23" s="8"/>
+      <c r="AO23" s="8"/>
+      <c r="AP23" s="8"/>
+      <c r="AQ23" s="8"/>
+      <c r="AR23" s="8"/>
+      <c r="AS23" s="8"/>
+      <c r="AT23" s="8"/>
+      <c r="AU23" s="8"/>
+      <c r="AV23" s="8"/>
+      <c r="AW23" s="8"/>
+      <c r="AX23" s="8"/>
+      <c r="AY23" s="8"/>
+      <c r="AZ23" s="8"/>
+      <c r="BA23" s="8"/>
+      <c r="BB23" s="8"/>
+      <c r="BC23" s="8"/>
+      <c r="BD23" s="8"/>
+      <c r="BE23" s="8"/>
+      <c r="BF23" s="8"/>
+      <c r="BG23" s="8"/>
+      <c r="BH23" s="8"/>
+      <c r="BI23" s="8"/>
+      <c r="BJ23" s="8"/>
+      <c r="BK23" s="8"/>
+      <c r="BL23" s="8"/>
+      <c r="BM23" s="8"/>
     </row>
-    <row r="24" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:65" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A24" s="1">
         <v>23</v>
       </c>
@@ -2816,8 +4980,94 @@
       <c r="Q24" s="5" t="s">
         <v>362</v>
       </c>
+      <c r="R24" s="7" t="s">
+        <v>369</v>
+      </c>
+      <c r="S24" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="T24" s="9">
+        <v>0.95</v>
+      </c>
+      <c r="U24" s="9">
+        <v>1</v>
+      </c>
+      <c r="V24" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="W24" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="X24" s="9">
+        <v>1</v>
+      </c>
+      <c r="Y24" s="9">
+        <v>1</v>
+      </c>
+      <c r="Z24" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AA24" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AB24" s="9">
+        <v>1</v>
+      </c>
+      <c r="AC24" s="9">
+        <v>0</v>
+      </c>
+      <c r="AD24" s="9">
+        <v>0</v>
+      </c>
+      <c r="AE24" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AF24" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AG24" s="9">
+        <v>0</v>
+      </c>
+      <c r="AH24" s="9">
+        <v>0</v>
+      </c>
+      <c r="AI24" s="9">
+        <v>0</v>
+      </c>
+      <c r="AJ24" s="9">
+        <v>0</v>
+      </c>
+      <c r="AK24" s="8"/>
+      <c r="AL24" s="8"/>
+      <c r="AM24" s="8"/>
+      <c r="AN24" s="8"/>
+      <c r="AO24" s="8"/>
+      <c r="AP24" s="8"/>
+      <c r="AQ24" s="8"/>
+      <c r="AR24" s="8"/>
+      <c r="AS24" s="8"/>
+      <c r="AT24" s="8"/>
+      <c r="AU24" s="8"/>
+      <c r="AV24" s="8"/>
+      <c r="AW24" s="8"/>
+      <c r="AX24" s="8"/>
+      <c r="AY24" s="8"/>
+      <c r="AZ24" s="8"/>
+      <c r="BA24" s="8"/>
+      <c r="BB24" s="8"/>
+      <c r="BC24" s="8"/>
+      <c r="BD24" s="8"/>
+      <c r="BE24" s="8"/>
+      <c r="BF24" s="8"/>
+      <c r="BG24" s="8"/>
+      <c r="BH24" s="8"/>
+      <c r="BI24" s="8"/>
+      <c r="BJ24" s="8"/>
+      <c r="BK24" s="8"/>
+      <c r="BL24" s="8"/>
+      <c r="BM24" s="8"/>
     </row>
-    <row r="25" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:65" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A25" s="1">
         <v>24</v>
       </c>
@@ -2869,8 +5119,94 @@
       <c r="Q25" s="5" t="s">
         <v>362</v>
       </c>
+      <c r="R25" s="7" t="s">
+        <v>390</v>
+      </c>
+      <c r="S25" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="T25" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="U25" s="9">
+        <v>1</v>
+      </c>
+      <c r="V25" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="W25" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="X25" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="Y25" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z25" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AA25" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AB25" s="9">
+        <v>0</v>
+      </c>
+      <c r="AC25" s="9">
+        <v>1</v>
+      </c>
+      <c r="AD25" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AE25" s="9">
+        <v>1</v>
+      </c>
+      <c r="AF25" s="9">
+        <v>0</v>
+      </c>
+      <c r="AG25" s="9">
+        <v>1</v>
+      </c>
+      <c r="AH25" s="9">
+        <v>0</v>
+      </c>
+      <c r="AI25" s="9">
+        <v>1</v>
+      </c>
+      <c r="AJ25" s="9">
+        <v>1</v>
+      </c>
+      <c r="AK25" s="8"/>
+      <c r="AL25" s="8"/>
+      <c r="AM25" s="8"/>
+      <c r="AN25" s="8"/>
+      <c r="AO25" s="8"/>
+      <c r="AP25" s="8"/>
+      <c r="AQ25" s="8"/>
+      <c r="AR25" s="8"/>
+      <c r="AS25" s="8"/>
+      <c r="AT25" s="8"/>
+      <c r="AU25" s="8"/>
+      <c r="AV25" s="8"/>
+      <c r="AW25" s="8"/>
+      <c r="AX25" s="8"/>
+      <c r="AY25" s="8"/>
+      <c r="AZ25" s="8"/>
+      <c r="BA25" s="8"/>
+      <c r="BB25" s="8"/>
+      <c r="BC25" s="8"/>
+      <c r="BD25" s="8"/>
+      <c r="BE25" s="8"/>
+      <c r="BF25" s="8"/>
+      <c r="BG25" s="8"/>
+      <c r="BH25" s="8"/>
+      <c r="BI25" s="8"/>
+      <c r="BJ25" s="8"/>
+      <c r="BK25" s="8"/>
+      <c r="BL25" s="8"/>
+      <c r="BM25" s="8"/>
     </row>
-    <row r="26" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:65" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A26" s="1">
         <v>25</v>
       </c>
@@ -2922,8 +5258,94 @@
       <c r="Q26" s="5" t="s">
         <v>363</v>
       </c>
+      <c r="R26" s="7" t="s">
+        <v>391</v>
+      </c>
+      <c r="S26" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="T26" s="9">
+        <v>0.8</v>
+      </c>
+      <c r="U26" s="9">
+        <v>1</v>
+      </c>
+      <c r="V26" s="9">
+        <v>0.8</v>
+      </c>
+      <c r="W26" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="X26" s="9">
+        <v>0</v>
+      </c>
+      <c r="Y26" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z26" s="9">
+        <v>0.8</v>
+      </c>
+      <c r="AA26" s="9">
+        <v>0.8</v>
+      </c>
+      <c r="AB26" s="9">
+        <v>1</v>
+      </c>
+      <c r="AC26" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AD26" s="9">
+        <v>0</v>
+      </c>
+      <c r="AE26" s="9">
+        <v>0</v>
+      </c>
+      <c r="AF26" s="9">
+        <v>0</v>
+      </c>
+      <c r="AG26" s="9">
+        <v>1</v>
+      </c>
+      <c r="AH26" s="9">
+        <v>0</v>
+      </c>
+      <c r="AI26" s="9">
+        <v>0</v>
+      </c>
+      <c r="AJ26" s="9">
+        <v>0</v>
+      </c>
+      <c r="AK26" s="8"/>
+      <c r="AL26" s="8"/>
+      <c r="AM26" s="8"/>
+      <c r="AN26" s="8"/>
+      <c r="AO26" s="8"/>
+      <c r="AP26" s="8"/>
+      <c r="AQ26" s="8"/>
+      <c r="AR26" s="8"/>
+      <c r="AS26" s="8"/>
+      <c r="AT26" s="8"/>
+      <c r="AU26" s="8"/>
+      <c r="AV26" s="8"/>
+      <c r="AW26" s="8"/>
+      <c r="AX26" s="8"/>
+      <c r="AY26" s="8"/>
+      <c r="AZ26" s="8"/>
+      <c r="BA26" s="8"/>
+      <c r="BB26" s="8"/>
+      <c r="BC26" s="8"/>
+      <c r="BD26" s="8"/>
+      <c r="BE26" s="8"/>
+      <c r="BF26" s="8"/>
+      <c r="BG26" s="8"/>
+      <c r="BH26" s="8"/>
+      <c r="BI26" s="8"/>
+      <c r="BJ26" s="8"/>
+      <c r="BK26" s="8"/>
+      <c r="BL26" s="8"/>
+      <c r="BM26" s="8"/>
     </row>
-    <row r="27" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:65" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A27" s="1">
         <v>26</v>
       </c>
@@ -2975,8 +5397,94 @@
       <c r="Q27" s="5" t="s">
         <v>362</v>
       </c>
+      <c r="R27" s="7" t="s">
+        <v>392</v>
+      </c>
+      <c r="S27" s="9">
+        <v>1</v>
+      </c>
+      <c r="T27" s="9">
+        <v>1</v>
+      </c>
+      <c r="U27" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="V27" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="W27" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="X27" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="Y27" s="9">
+        <v>0.8</v>
+      </c>
+      <c r="Z27" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="AA27" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="AB27" s="9">
+        <v>1</v>
+      </c>
+      <c r="AC27" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="AD27" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="AE27" s="9">
+        <v>1</v>
+      </c>
+      <c r="AF27" s="9">
+        <v>1</v>
+      </c>
+      <c r="AG27" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AH27" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AI27" s="9">
+        <v>0</v>
+      </c>
+      <c r="AJ27" s="9">
+        <v>0</v>
+      </c>
+      <c r="AK27" s="8"/>
+      <c r="AL27" s="8"/>
+      <c r="AM27" s="8"/>
+      <c r="AN27" s="8"/>
+      <c r="AO27" s="8"/>
+      <c r="AP27" s="8"/>
+      <c r="AQ27" s="8"/>
+      <c r="AR27" s="8"/>
+      <c r="AS27" s="8"/>
+      <c r="AT27" s="8"/>
+      <c r="AU27" s="8"/>
+      <c r="AV27" s="8"/>
+      <c r="AW27" s="8"/>
+      <c r="AX27" s="8"/>
+      <c r="AY27" s="8"/>
+      <c r="AZ27" s="8"/>
+      <c r="BA27" s="8"/>
+      <c r="BB27" s="8"/>
+      <c r="BC27" s="8"/>
+      <c r="BD27" s="8"/>
+      <c r="BE27" s="8"/>
+      <c r="BF27" s="8"/>
+      <c r="BG27" s="8"/>
+      <c r="BH27" s="8"/>
+      <c r="BI27" s="8"/>
+      <c r="BJ27" s="8"/>
+      <c r="BK27" s="8"/>
+      <c r="BL27" s="8"/>
+      <c r="BM27" s="8"/>
     </row>
-    <row r="28" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:65" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A28" s="1">
         <v>27</v>
       </c>
@@ -3028,8 +5536,94 @@
       <c r="Q28" s="5" t="s">
         <v>363</v>
       </c>
+      <c r="R28" s="7" t="s">
+        <v>393</v>
+      </c>
+      <c r="S28" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="T28" s="9">
+        <v>0.6</v>
+      </c>
+      <c r="U28" s="9">
+        <v>1</v>
+      </c>
+      <c r="V28" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="W28" s="9">
+        <v>0</v>
+      </c>
+      <c r="X28" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="Y28" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z28" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AA28" s="9">
+        <v>0</v>
+      </c>
+      <c r="AB28" s="9">
+        <v>1</v>
+      </c>
+      <c r="AC28" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AD28" s="9">
+        <v>0</v>
+      </c>
+      <c r="AE28" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AF28" s="9">
+        <v>0</v>
+      </c>
+      <c r="AG28" s="9">
+        <v>0</v>
+      </c>
+      <c r="AH28" s="9">
+        <v>0</v>
+      </c>
+      <c r="AI28" s="9">
+        <v>0</v>
+      </c>
+      <c r="AJ28" s="9">
+        <v>0</v>
+      </c>
+      <c r="AK28" s="8"/>
+      <c r="AL28" s="8"/>
+      <c r="AM28" s="8"/>
+      <c r="AN28" s="8"/>
+      <c r="AO28" s="8"/>
+      <c r="AP28" s="8"/>
+      <c r="AQ28" s="8"/>
+      <c r="AR28" s="8"/>
+      <c r="AS28" s="8"/>
+      <c r="AT28" s="8"/>
+      <c r="AU28" s="8"/>
+      <c r="AV28" s="8"/>
+      <c r="AW28" s="8"/>
+      <c r="AX28" s="8"/>
+      <c r="AY28" s="8"/>
+      <c r="AZ28" s="8"/>
+      <c r="BA28" s="8"/>
+      <c r="BB28" s="8"/>
+      <c r="BC28" s="8"/>
+      <c r="BD28" s="8"/>
+      <c r="BE28" s="8"/>
+      <c r="BF28" s="8"/>
+      <c r="BG28" s="8"/>
+      <c r="BH28" s="8"/>
+      <c r="BI28" s="8"/>
+      <c r="BJ28" s="8"/>
+      <c r="BK28" s="8"/>
+      <c r="BL28" s="8"/>
+      <c r="BM28" s="8"/>
     </row>
-    <row r="29" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:65" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A29" s="1">
         <v>28</v>
       </c>
@@ -3081,8 +5675,94 @@
       <c r="Q29" s="5" t="s">
         <v>362</v>
       </c>
+      <c r="R29" s="7" t="s">
+        <v>394</v>
+      </c>
+      <c r="S29" s="9">
+        <v>1</v>
+      </c>
+      <c r="T29" s="9">
+        <v>1</v>
+      </c>
+      <c r="U29" s="9">
+        <v>1</v>
+      </c>
+      <c r="V29" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="W29" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="X29" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="Y29" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="Z29" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="AA29" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="AB29" s="9">
+        <v>1</v>
+      </c>
+      <c r="AC29" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="AD29" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="AE29" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AF29" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AG29" s="9">
+        <v>0</v>
+      </c>
+      <c r="AH29" s="9">
+        <v>0</v>
+      </c>
+      <c r="AI29" s="9">
+        <v>0</v>
+      </c>
+      <c r="AJ29" s="9">
+        <v>0</v>
+      </c>
+      <c r="AK29" s="8"/>
+      <c r="AL29" s="8"/>
+      <c r="AM29" s="8"/>
+      <c r="AN29" s="8"/>
+      <c r="AO29" s="8"/>
+      <c r="AP29" s="8"/>
+      <c r="AQ29" s="8"/>
+      <c r="AR29" s="8"/>
+      <c r="AS29" s="8"/>
+      <c r="AT29" s="8"/>
+      <c r="AU29" s="8"/>
+      <c r="AV29" s="8"/>
+      <c r="AW29" s="8"/>
+      <c r="AX29" s="8"/>
+      <c r="AY29" s="8"/>
+      <c r="AZ29" s="8"/>
+      <c r="BA29" s="8"/>
+      <c r="BB29" s="8"/>
+      <c r="BC29" s="8"/>
+      <c r="BD29" s="8"/>
+      <c r="BE29" s="8"/>
+      <c r="BF29" s="8"/>
+      <c r="BG29" s="8"/>
+      <c r="BH29" s="8"/>
+      <c r="BI29" s="8"/>
+      <c r="BJ29" s="8"/>
+      <c r="BK29" s="8"/>
+      <c r="BL29" s="8"/>
+      <c r="BM29" s="8"/>
     </row>
-    <row r="30" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:65" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A30" s="1">
         <v>29</v>
       </c>
@@ -3134,8 +5814,94 @@
       <c r="Q30" s="5" t="s">
         <v>363</v>
       </c>
+      <c r="R30" s="7" t="s">
+        <v>367</v>
+      </c>
+      <c r="S30" s="9">
+        <v>1</v>
+      </c>
+      <c r="T30" s="9">
+        <v>0.41</v>
+      </c>
+      <c r="U30" s="9">
+        <v>1</v>
+      </c>
+      <c r="V30" s="9">
+        <v>0.8</v>
+      </c>
+      <c r="W30" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="X30" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="Y30" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z30" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="AA30" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="AB30" s="9">
+        <v>0</v>
+      </c>
+      <c r="AC30" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="AD30" s="9">
+        <v>0.41</v>
+      </c>
+      <c r="AE30" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="AF30" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="AG30" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="AH30" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="AI30" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="AJ30" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="AK30" s="8"/>
+      <c r="AL30" s="8"/>
+      <c r="AM30" s="8"/>
+      <c r="AN30" s="8"/>
+      <c r="AO30" s="8"/>
+      <c r="AP30" s="8"/>
+      <c r="AQ30" s="8"/>
+      <c r="AR30" s="8"/>
+      <c r="AS30" s="8"/>
+      <c r="AT30" s="8"/>
+      <c r="AU30" s="8"/>
+      <c r="AV30" s="8"/>
+      <c r="AW30" s="8"/>
+      <c r="AX30" s="8"/>
+      <c r="AY30" s="8"/>
+      <c r="AZ30" s="8"/>
+      <c r="BA30" s="8"/>
+      <c r="BB30" s="8"/>
+      <c r="BC30" s="8"/>
+      <c r="BD30" s="8"/>
+      <c r="BE30" s="8"/>
+      <c r="BF30" s="8"/>
+      <c r="BG30" s="8"/>
+      <c r="BH30" s="8"/>
+      <c r="BI30" s="8"/>
+      <c r="BJ30" s="8"/>
+      <c r="BK30" s="8"/>
+      <c r="BL30" s="8"/>
+      <c r="BM30" s="8"/>
     </row>
-    <row r="31" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:65" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A31" s="1">
         <v>30</v>
       </c>
@@ -3187,8 +5953,94 @@
       <c r="Q31" s="5" t="s">
         <v>362</v>
       </c>
+      <c r="R31" s="7" t="s">
+        <v>395</v>
+      </c>
+      <c r="S31" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="T31" s="9">
+        <v>0</v>
+      </c>
+      <c r="U31" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="V31" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="W31" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="X31" s="9">
+        <v>1</v>
+      </c>
+      <c r="Y31" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z31" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="AA31" s="9">
+        <v>0</v>
+      </c>
+      <c r="AB31" s="9">
+        <v>1</v>
+      </c>
+      <c r="AC31" s="9">
+        <v>1</v>
+      </c>
+      <c r="AD31" s="9">
+        <v>0</v>
+      </c>
+      <c r="AE31" s="9">
+        <v>1</v>
+      </c>
+      <c r="AF31" s="9">
+        <v>0</v>
+      </c>
+      <c r="AG31" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AH31" s="9">
+        <v>0</v>
+      </c>
+      <c r="AI31" s="9">
+        <v>0</v>
+      </c>
+      <c r="AJ31" s="9">
+        <v>0</v>
+      </c>
+      <c r="AK31" s="8"/>
+      <c r="AL31" s="8"/>
+      <c r="AM31" s="8"/>
+      <c r="AN31" s="8"/>
+      <c r="AO31" s="8"/>
+      <c r="AP31" s="8"/>
+      <c r="AQ31" s="8"/>
+      <c r="AR31" s="8"/>
+      <c r="AS31" s="8"/>
+      <c r="AT31" s="8"/>
+      <c r="AU31" s="8"/>
+      <c r="AV31" s="8"/>
+      <c r="AW31" s="8"/>
+      <c r="AX31" s="8"/>
+      <c r="AY31" s="8"/>
+      <c r="AZ31" s="8"/>
+      <c r="BA31" s="8"/>
+      <c r="BB31" s="8"/>
+      <c r="BC31" s="8"/>
+      <c r="BD31" s="8"/>
+      <c r="BE31" s="8"/>
+      <c r="BF31" s="8"/>
+      <c r="BG31" s="8"/>
+      <c r="BH31" s="8"/>
+      <c r="BI31" s="8"/>
+      <c r="BJ31" s="8"/>
+      <c r="BK31" s="8"/>
+      <c r="BL31" s="8"/>
+      <c r="BM31" s="8"/>
     </row>
-    <row r="32" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:65" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A32" s="1">
         <v>31</v>
       </c>
@@ -3240,8 +6092,94 @@
       <c r="Q32" s="5" t="s">
         <v>363</v>
       </c>
+      <c r="R32" s="7" t="s">
+        <v>396</v>
+      </c>
+      <c r="S32" s="9">
+        <v>1</v>
+      </c>
+      <c r="T32" s="9">
+        <v>1</v>
+      </c>
+      <c r="U32" s="9">
+        <v>0.8</v>
+      </c>
+      <c r="V32" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="W32" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="X32" s="9">
+        <v>1</v>
+      </c>
+      <c r="Y32" s="9">
+        <v>1</v>
+      </c>
+      <c r="Z32" s="9">
+        <v>1</v>
+      </c>
+      <c r="AA32" s="9">
+        <v>1</v>
+      </c>
+      <c r="AB32" s="9">
+        <v>1</v>
+      </c>
+      <c r="AC32" s="9">
+        <v>1</v>
+      </c>
+      <c r="AD32" s="9">
+        <v>1</v>
+      </c>
+      <c r="AE32" s="9">
+        <v>0.05</v>
+      </c>
+      <c r="AF32" s="9">
+        <v>0.05</v>
+      </c>
+      <c r="AG32" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AH32" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AI32" s="9">
+        <v>0</v>
+      </c>
+      <c r="AJ32" s="9">
+        <v>0</v>
+      </c>
+      <c r="AK32" s="8"/>
+      <c r="AL32" s="8"/>
+      <c r="AM32" s="8"/>
+      <c r="AN32" s="8"/>
+      <c r="AO32" s="8"/>
+      <c r="AP32" s="8"/>
+      <c r="AQ32" s="8"/>
+      <c r="AR32" s="8"/>
+      <c r="AS32" s="8"/>
+      <c r="AT32" s="8"/>
+      <c r="AU32" s="8"/>
+      <c r="AV32" s="8"/>
+      <c r="AW32" s="8"/>
+      <c r="AX32" s="8"/>
+      <c r="AY32" s="8"/>
+      <c r="AZ32" s="8"/>
+      <c r="BA32" s="8"/>
+      <c r="BB32" s="8"/>
+      <c r="BC32" s="8"/>
+      <c r="BD32" s="8"/>
+      <c r="BE32" s="8"/>
+      <c r="BF32" s="8"/>
+      <c r="BG32" s="8"/>
+      <c r="BH32" s="8"/>
+      <c r="BI32" s="8"/>
+      <c r="BJ32" s="8"/>
+      <c r="BK32" s="8"/>
+      <c r="BL32" s="8"/>
+      <c r="BM32" s="8"/>
     </row>
-    <row r="33" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:65" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A33" s="1">
         <v>32</v>
       </c>
@@ -3293,8 +6231,94 @@
       <c r="Q33" s="5" t="s">
         <v>363</v>
       </c>
+      <c r="R33" s="7" t="s">
+        <v>397</v>
+      </c>
+      <c r="S33" s="9">
+        <v>1</v>
+      </c>
+      <c r="T33" s="9">
+        <v>1</v>
+      </c>
+      <c r="U33" s="9">
+        <v>0.8</v>
+      </c>
+      <c r="V33" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="W33" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="X33" s="9">
+        <v>1</v>
+      </c>
+      <c r="Y33" s="9">
+        <v>1</v>
+      </c>
+      <c r="Z33" s="9">
+        <v>1</v>
+      </c>
+      <c r="AA33" s="9">
+        <v>1</v>
+      </c>
+      <c r="AB33" s="9">
+        <v>1</v>
+      </c>
+      <c r="AC33" s="9">
+        <v>1</v>
+      </c>
+      <c r="AD33" s="9">
+        <v>1</v>
+      </c>
+      <c r="AE33" s="9">
+        <v>0.05</v>
+      </c>
+      <c r="AF33" s="9">
+        <v>0.05</v>
+      </c>
+      <c r="AG33" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AH33" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AI33" s="9">
+        <v>0</v>
+      </c>
+      <c r="AJ33" s="9">
+        <v>0</v>
+      </c>
+      <c r="AK33" s="8"/>
+      <c r="AL33" s="8"/>
+      <c r="AM33" s="8"/>
+      <c r="AN33" s="8"/>
+      <c r="AO33" s="8"/>
+      <c r="AP33" s="8"/>
+      <c r="AQ33" s="8"/>
+      <c r="AR33" s="8"/>
+      <c r="AS33" s="8"/>
+      <c r="AT33" s="8"/>
+      <c r="AU33" s="8"/>
+      <c r="AV33" s="8"/>
+      <c r="AW33" s="8"/>
+      <c r="AX33" s="8"/>
+      <c r="AY33" s="8"/>
+      <c r="AZ33" s="8"/>
+      <c r="BA33" s="8"/>
+      <c r="BB33" s="8"/>
+      <c r="BC33" s="8"/>
+      <c r="BD33" s="8"/>
+      <c r="BE33" s="8"/>
+      <c r="BF33" s="8"/>
+      <c r="BG33" s="8"/>
+      <c r="BH33" s="8"/>
+      <c r="BI33" s="8"/>
+      <c r="BJ33" s="8"/>
+      <c r="BK33" s="8"/>
+      <c r="BL33" s="8"/>
+      <c r="BM33" s="8"/>
     </row>
-    <row r="34" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:65" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A34" s="1">
         <v>33</v>
       </c>
@@ -3346,8 +6370,94 @@
       <c r="Q34" s="5" t="s">
         <v>363</v>
       </c>
+      <c r="R34" s="7" t="s">
+        <v>398</v>
+      </c>
+      <c r="S34" s="9">
+        <v>1</v>
+      </c>
+      <c r="T34" s="9">
+        <v>1</v>
+      </c>
+      <c r="U34" s="9">
+        <v>0.8</v>
+      </c>
+      <c r="V34" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="W34" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="X34" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="Y34" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="Z34" s="9">
+        <v>1</v>
+      </c>
+      <c r="AA34" s="9">
+        <v>1</v>
+      </c>
+      <c r="AB34" s="9">
+        <v>1</v>
+      </c>
+      <c r="AC34" s="9">
+        <v>1</v>
+      </c>
+      <c r="AD34" s="9">
+        <v>1</v>
+      </c>
+      <c r="AE34" s="9">
+        <v>0.05</v>
+      </c>
+      <c r="AF34" s="9">
+        <v>0.05</v>
+      </c>
+      <c r="AG34" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AH34" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AI34" s="9">
+        <v>0</v>
+      </c>
+      <c r="AJ34" s="9">
+        <v>0</v>
+      </c>
+      <c r="AK34" s="8"/>
+      <c r="AL34" s="8"/>
+      <c r="AM34" s="8"/>
+      <c r="AN34" s="8"/>
+      <c r="AO34" s="8"/>
+      <c r="AP34" s="8"/>
+      <c r="AQ34" s="8"/>
+      <c r="AR34" s="8"/>
+      <c r="AS34" s="8"/>
+      <c r="AT34" s="8"/>
+      <c r="AU34" s="8"/>
+      <c r="AV34" s="8"/>
+      <c r="AW34" s="8"/>
+      <c r="AX34" s="8"/>
+      <c r="AY34" s="8"/>
+      <c r="AZ34" s="8"/>
+      <c r="BA34" s="8"/>
+      <c r="BB34" s="8"/>
+      <c r="BC34" s="8"/>
+      <c r="BD34" s="8"/>
+      <c r="BE34" s="8"/>
+      <c r="BF34" s="8"/>
+      <c r="BG34" s="8"/>
+      <c r="BH34" s="8"/>
+      <c r="BI34" s="8"/>
+      <c r="BJ34" s="8"/>
+      <c r="BK34" s="8"/>
+      <c r="BL34" s="8"/>
+      <c r="BM34" s="8"/>
     </row>
-    <row r="35" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:65" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A35" s="1">
         <v>34</v>
       </c>
@@ -3399,8 +6509,94 @@
       <c r="Q35" s="5" t="s">
         <v>363</v>
       </c>
+      <c r="R35" s="7" t="s">
+        <v>399</v>
+      </c>
+      <c r="S35" s="9">
+        <v>1</v>
+      </c>
+      <c r="T35" s="9">
+        <v>0</v>
+      </c>
+      <c r="U35" s="9">
+        <v>1</v>
+      </c>
+      <c r="V35" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="W35" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="X35" s="9">
+        <v>0.8</v>
+      </c>
+      <c r="Y35" s="9">
+        <v>1</v>
+      </c>
+      <c r="Z35" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="AA35" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="AB35" s="9">
+        <v>0</v>
+      </c>
+      <c r="AC35" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="AD35" s="9">
+        <v>0</v>
+      </c>
+      <c r="AE35" s="9">
+        <v>0.8</v>
+      </c>
+      <c r="AF35" s="9">
+        <v>0.8</v>
+      </c>
+      <c r="AG35" s="9">
+        <v>1</v>
+      </c>
+      <c r="AH35" s="9">
+        <v>1</v>
+      </c>
+      <c r="AI35" s="9">
+        <v>0.8</v>
+      </c>
+      <c r="AJ35" s="9">
+        <v>0.8</v>
+      </c>
+      <c r="AK35" s="8"/>
+      <c r="AL35" s="8"/>
+      <c r="AM35" s="8"/>
+      <c r="AN35" s="8"/>
+      <c r="AO35" s="8"/>
+      <c r="AP35" s="8"/>
+      <c r="AQ35" s="8"/>
+      <c r="AR35" s="8"/>
+      <c r="AS35" s="8"/>
+      <c r="AT35" s="8"/>
+      <c r="AU35" s="8"/>
+      <c r="AV35" s="8"/>
+      <c r="AW35" s="8"/>
+      <c r="AX35" s="8"/>
+      <c r="AY35" s="8"/>
+      <c r="AZ35" s="8"/>
+      <c r="BA35" s="8"/>
+      <c r="BB35" s="8"/>
+      <c r="BC35" s="8"/>
+      <c r="BD35" s="8"/>
+      <c r="BE35" s="8"/>
+      <c r="BF35" s="8"/>
+      <c r="BG35" s="8"/>
+      <c r="BH35" s="8"/>
+      <c r="BI35" s="8"/>
+      <c r="BJ35" s="8"/>
+      <c r="BK35" s="8"/>
+      <c r="BL35" s="8"/>
+      <c r="BM35" s="8"/>
     </row>
-    <row r="36" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:65" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A36" s="1">
         <v>35</v>
       </c>
@@ -3452,8 +6648,94 @@
       <c r="Q36" s="5" t="s">
         <v>363</v>
       </c>
+      <c r="R36" s="7" t="s">
+        <v>400</v>
+      </c>
+      <c r="S36" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="T36" s="9">
+        <v>0.3</v>
+      </c>
+      <c r="U36" s="9">
+        <v>1</v>
+      </c>
+      <c r="V36" s="9">
+        <v>0.8</v>
+      </c>
+      <c r="W36" s="9">
+        <v>0</v>
+      </c>
+      <c r="X36" s="9">
+        <v>0</v>
+      </c>
+      <c r="Y36" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z36" s="9">
+        <v>0</v>
+      </c>
+      <c r="AA36" s="9">
+        <v>0</v>
+      </c>
+      <c r="AB36" s="9">
+        <v>1</v>
+      </c>
+      <c r="AC36" s="9">
+        <v>0</v>
+      </c>
+      <c r="AD36" s="9">
+        <v>0</v>
+      </c>
+      <c r="AE36" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AF36" s="9">
+        <v>0</v>
+      </c>
+      <c r="AG36" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AH36" s="9">
+        <v>0</v>
+      </c>
+      <c r="AI36" s="9">
+        <v>0</v>
+      </c>
+      <c r="AJ36" s="9">
+        <v>0</v>
+      </c>
+      <c r="AK36" s="8"/>
+      <c r="AL36" s="8"/>
+      <c r="AM36" s="8"/>
+      <c r="AN36" s="8"/>
+      <c r="AO36" s="8"/>
+      <c r="AP36" s="8"/>
+      <c r="AQ36" s="8"/>
+      <c r="AR36" s="8"/>
+      <c r="AS36" s="8"/>
+      <c r="AT36" s="8"/>
+      <c r="AU36" s="8"/>
+      <c r="AV36" s="8"/>
+      <c r="AW36" s="8"/>
+      <c r="AX36" s="8"/>
+      <c r="AY36" s="8"/>
+      <c r="AZ36" s="8"/>
+      <c r="BA36" s="8"/>
+      <c r="BB36" s="8"/>
+      <c r="BC36" s="8"/>
+      <c r="BD36" s="8"/>
+      <c r="BE36" s="8"/>
+      <c r="BF36" s="8"/>
+      <c r="BG36" s="8"/>
+      <c r="BH36" s="8"/>
+      <c r="BI36" s="8"/>
+      <c r="BJ36" s="8"/>
+      <c r="BK36" s="8"/>
+      <c r="BL36" s="8"/>
+      <c r="BM36" s="8"/>
     </row>
-    <row r="37" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:65" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A37" s="1">
         <v>36</v>
       </c>
@@ -3505,8 +6787,94 @@
       <c r="Q37" s="5" t="s">
         <v>363</v>
       </c>
+      <c r="R37" s="7" t="s">
+        <v>401</v>
+      </c>
+      <c r="S37" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="T37" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="U37" s="9">
+        <v>0</v>
+      </c>
+      <c r="V37" s="9">
+        <v>0</v>
+      </c>
+      <c r="W37" s="9">
+        <v>0</v>
+      </c>
+      <c r="X37" s="9">
+        <v>0</v>
+      </c>
+      <c r="Y37" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z37" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AA37" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AB37" s="9">
+        <v>1</v>
+      </c>
+      <c r="AC37" s="9">
+        <v>1</v>
+      </c>
+      <c r="AD37" s="9">
+        <v>1</v>
+      </c>
+      <c r="AE37" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AF37" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AG37" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AH37" s="9">
+        <v>0</v>
+      </c>
+      <c r="AI37" s="9">
+        <v>0</v>
+      </c>
+      <c r="AJ37" s="9">
+        <v>0</v>
+      </c>
+      <c r="AK37" s="8"/>
+      <c r="AL37" s="8"/>
+      <c r="AM37" s="8"/>
+      <c r="AN37" s="8"/>
+      <c r="AO37" s="8"/>
+      <c r="AP37" s="8"/>
+      <c r="AQ37" s="8"/>
+      <c r="AR37" s="8"/>
+      <c r="AS37" s="8"/>
+      <c r="AT37" s="8"/>
+      <c r="AU37" s="8"/>
+      <c r="AV37" s="8"/>
+      <c r="AW37" s="8"/>
+      <c r="AX37" s="8"/>
+      <c r="AY37" s="8"/>
+      <c r="AZ37" s="8"/>
+      <c r="BA37" s="8"/>
+      <c r="BB37" s="8"/>
+      <c r="BC37" s="8"/>
+      <c r="BD37" s="8"/>
+      <c r="BE37" s="8"/>
+      <c r="BF37" s="8"/>
+      <c r="BG37" s="8"/>
+      <c r="BH37" s="8"/>
+      <c r="BI37" s="8"/>
+      <c r="BJ37" s="8"/>
+      <c r="BK37" s="8"/>
+      <c r="BL37" s="8"/>
+      <c r="BM37" s="8"/>
     </row>
-    <row r="38" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:65" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A38" s="1">
         <v>37</v>
       </c>
@@ -3558,8 +6926,94 @@
       <c r="Q38" s="5" t="s">
         <v>363</v>
       </c>
+      <c r="R38" s="7" t="s">
+        <v>402</v>
+      </c>
+      <c r="S38" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="T38" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="U38" s="9">
+        <v>0</v>
+      </c>
+      <c r="V38" s="9">
+        <v>0</v>
+      </c>
+      <c r="W38" s="9">
+        <v>0</v>
+      </c>
+      <c r="X38" s="9">
+        <v>0</v>
+      </c>
+      <c r="Y38" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z38" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AA38" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AB38" s="9">
+        <v>1</v>
+      </c>
+      <c r="AC38" s="9">
+        <v>1</v>
+      </c>
+      <c r="AD38" s="9">
+        <v>1</v>
+      </c>
+      <c r="AE38" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AF38" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AG38" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AH38" s="9">
+        <v>0</v>
+      </c>
+      <c r="AI38" s="9">
+        <v>0</v>
+      </c>
+      <c r="AJ38" s="9">
+        <v>0</v>
+      </c>
+      <c r="AK38" s="8"/>
+      <c r="AL38" s="8"/>
+      <c r="AM38" s="8"/>
+      <c r="AN38" s="8"/>
+      <c r="AO38" s="8"/>
+      <c r="AP38" s="8"/>
+      <c r="AQ38" s="8"/>
+      <c r="AR38" s="8"/>
+      <c r="AS38" s="8"/>
+      <c r="AT38" s="8"/>
+      <c r="AU38" s="8"/>
+      <c r="AV38" s="8"/>
+      <c r="AW38" s="8"/>
+      <c r="AX38" s="8"/>
+      <c r="AY38" s="8"/>
+      <c r="AZ38" s="8"/>
+      <c r="BA38" s="8"/>
+      <c r="BB38" s="8"/>
+      <c r="BC38" s="8"/>
+      <c r="BD38" s="8"/>
+      <c r="BE38" s="8"/>
+      <c r="BF38" s="8"/>
+      <c r="BG38" s="8"/>
+      <c r="BH38" s="8"/>
+      <c r="BI38" s="8"/>
+      <c r="BJ38" s="8"/>
+      <c r="BK38" s="8"/>
+      <c r="BL38" s="8"/>
+      <c r="BM38" s="8"/>
     </row>
-    <row r="39" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:65" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A39" s="1">
         <v>38</v>
       </c>
@@ -3611,8 +7065,94 @@
       <c r="Q39" s="5" t="s">
         <v>363</v>
       </c>
+      <c r="R39" s="7" t="s">
+        <v>403</v>
+      </c>
+      <c r="S39" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="T39" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="U39" s="9">
+        <v>0</v>
+      </c>
+      <c r="V39" s="9">
+        <v>0</v>
+      </c>
+      <c r="W39" s="9">
+        <v>0</v>
+      </c>
+      <c r="X39" s="9">
+        <v>0</v>
+      </c>
+      <c r="Y39" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z39" s="9">
+        <v>0.8</v>
+      </c>
+      <c r="AA39" s="9">
+        <v>0.8</v>
+      </c>
+      <c r="AB39" s="9">
+        <v>1</v>
+      </c>
+      <c r="AC39" s="9">
+        <v>1</v>
+      </c>
+      <c r="AD39" s="9">
+        <v>1</v>
+      </c>
+      <c r="AE39" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AF39" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AG39" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AH39" s="9">
+        <v>0</v>
+      </c>
+      <c r="AI39" s="9">
+        <v>0</v>
+      </c>
+      <c r="AJ39" s="9">
+        <v>0</v>
+      </c>
+      <c r="AK39" s="8"/>
+      <c r="AL39" s="8"/>
+      <c r="AM39" s="8"/>
+      <c r="AN39" s="8"/>
+      <c r="AO39" s="8"/>
+      <c r="AP39" s="8"/>
+      <c r="AQ39" s="8"/>
+      <c r="AR39" s="8"/>
+      <c r="AS39" s="8"/>
+      <c r="AT39" s="8"/>
+      <c r="AU39" s="8"/>
+      <c r="AV39" s="8"/>
+      <c r="AW39" s="8"/>
+      <c r="AX39" s="8"/>
+      <c r="AY39" s="8"/>
+      <c r="AZ39" s="8"/>
+      <c r="BA39" s="8"/>
+      <c r="BB39" s="8"/>
+      <c r="BC39" s="8"/>
+      <c r="BD39" s="8"/>
+      <c r="BE39" s="8"/>
+      <c r="BF39" s="8"/>
+      <c r="BG39" s="8"/>
+      <c r="BH39" s="8"/>
+      <c r="BI39" s="8"/>
+      <c r="BJ39" s="8"/>
+      <c r="BK39" s="8"/>
+      <c r="BL39" s="8"/>
+      <c r="BM39" s="8"/>
     </row>
-    <row r="40" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:65" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A40" s="1">
         <v>39</v>
       </c>
@@ -3664,8 +7204,94 @@
       <c r="Q40" s="5" t="s">
         <v>363</v>
       </c>
+      <c r="R40" s="7" t="s">
+        <v>404</v>
+      </c>
+      <c r="S40" s="9">
+        <v>0.3</v>
+      </c>
+      <c r="T40" s="9">
+        <v>0</v>
+      </c>
+      <c r="U40" s="9">
+        <v>0</v>
+      </c>
+      <c r="V40" s="9">
+        <v>0</v>
+      </c>
+      <c r="W40" s="9">
+        <v>0</v>
+      </c>
+      <c r="X40" s="9">
+        <v>0</v>
+      </c>
+      <c r="Y40" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z40" s="9">
+        <v>0</v>
+      </c>
+      <c r="AA40" s="9">
+        <v>0</v>
+      </c>
+      <c r="AB40" s="9">
+        <v>1</v>
+      </c>
+      <c r="AC40" s="9">
+        <v>0</v>
+      </c>
+      <c r="AD40" s="9">
+        <v>0</v>
+      </c>
+      <c r="AE40" s="9">
+        <v>0</v>
+      </c>
+      <c r="AF40" s="9">
+        <v>0</v>
+      </c>
+      <c r="AG40" s="9">
+        <v>0</v>
+      </c>
+      <c r="AH40" s="9">
+        <v>0</v>
+      </c>
+      <c r="AI40" s="9">
+        <v>0</v>
+      </c>
+      <c r="AJ40" s="9">
+        <v>0</v>
+      </c>
+      <c r="AK40" s="8"/>
+      <c r="AL40" s="8"/>
+      <c r="AM40" s="8"/>
+      <c r="AN40" s="8"/>
+      <c r="AO40" s="8"/>
+      <c r="AP40" s="8"/>
+      <c r="AQ40" s="8"/>
+      <c r="AR40" s="8"/>
+      <c r="AS40" s="8"/>
+      <c r="AT40" s="8"/>
+      <c r="AU40" s="8"/>
+      <c r="AV40" s="8"/>
+      <c r="AW40" s="8"/>
+      <c r="AX40" s="8"/>
+      <c r="AY40" s="8"/>
+      <c r="AZ40" s="8"/>
+      <c r="BA40" s="8"/>
+      <c r="BB40" s="8"/>
+      <c r="BC40" s="8"/>
+      <c r="BD40" s="8"/>
+      <c r="BE40" s="8"/>
+      <c r="BF40" s="8"/>
+      <c r="BG40" s="8"/>
+      <c r="BH40" s="8"/>
+      <c r="BI40" s="8"/>
+      <c r="BJ40" s="8"/>
+      <c r="BK40" s="8"/>
+      <c r="BL40" s="8"/>
+      <c r="BM40" s="8"/>
     </row>
-    <row r="41" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:65" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A41" s="1">
         <v>40</v>
       </c>
@@ -3717,14 +7343,96 @@
       <c r="Q41" s="5" t="s">
         <v>363</v>
       </c>
+      <c r="R41" s="7" t="s">
+        <v>405</v>
+      </c>
+      <c r="S41" s="9">
+        <v>1</v>
+      </c>
+      <c r="T41" s="9">
+        <v>1</v>
+      </c>
+      <c r="U41" s="9">
+        <v>1</v>
+      </c>
+      <c r="V41" s="9">
+        <v>1</v>
+      </c>
+      <c r="W41" s="9">
+        <v>1</v>
+      </c>
+      <c r="X41" s="9">
+        <v>1</v>
+      </c>
+      <c r="Y41" s="9">
+        <v>1</v>
+      </c>
+      <c r="Z41" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="AA41" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="AB41" s="9">
+        <v>1</v>
+      </c>
+      <c r="AC41" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="AD41" s="9">
+        <v>0.9</v>
+      </c>
+      <c r="AE41" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AF41" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AG41" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AH41" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AI41" s="9">
+        <v>0</v>
+      </c>
+      <c r="AJ41" s="9">
+        <v>0</v>
+      </c>
+      <c r="AK41" s="8"/>
+      <c r="AL41" s="8"/>
+      <c r="AM41" s="8"/>
+      <c r="AN41" s="8"/>
+      <c r="AO41" s="8"/>
+      <c r="AP41" s="8"/>
+      <c r="AQ41" s="8"/>
+      <c r="AR41" s="8"/>
+      <c r="AS41" s="8"/>
+      <c r="AT41" s="8"/>
+      <c r="AU41" s="8"/>
+      <c r="AV41" s="8"/>
+      <c r="AW41" s="8"/>
+      <c r="AX41" s="8"/>
+      <c r="AY41" s="8"/>
+      <c r="AZ41" s="8"/>
+      <c r="BA41" s="8"/>
+      <c r="BB41" s="8"/>
+      <c r="BC41" s="8"/>
+      <c r="BD41" s="8"/>
+      <c r="BE41" s="8"/>
+      <c r="BF41" s="8"/>
+      <c r="BG41" s="8"/>
+      <c r="BH41" s="8"/>
+      <c r="BI41" s="8"/>
+      <c r="BJ41" s="8"/>
+      <c r="BK41" s="8"/>
+      <c r="BL41" s="8"/>
+      <c r="BM41" s="8"/>
     </row>
-    <row r="42" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="42" spans="1:65" s="5" customFormat="1" x14ac:dyDescent="0.4"/>
   </sheetData>
-  <autoFilter ref="A1:Q1" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:Q41">
-      <sortCondition ref="A1"/>
-    </sortState>
-  </autoFilter>
+  <autoFilter ref="A1:R1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3732,106 +7440,106 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:A21"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.15234375" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="100" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" ht="15.45" x14ac:dyDescent="0.4">
       <c r="A1" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A2" s="3"/>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A3" s="3" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A4" s="3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A5" s="3" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A6" s="3" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A7" s="3"/>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A8" s="4" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A9" s="3" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A10" s="3" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A11" s="3" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A12" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A13" s="3" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A14" s="3" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A15" s="3" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A16" s="3" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A17" s="3" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A18" s="3" t="s">
         <v>364</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A19" s="3"/>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A20" s="3" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A21" s="3" t="s">
         <v>34</v>
       </c>

</xml_diff>

<commit_message>
Mixtos: el CAPEX compartido de Concepción Mendizábal cuenta una vez
- Excel: las fases I, II y III llevan el CAPEX único de las tres
  ($925,310,833.00) en lugar de uno por fase.
- Resumen: en el CAPEX total, los proyectos del mismo socio con
  exactamente el mismo CAPEX cuentan una sola vez (kpis.js, con prueba).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01APiq7bAy76yveceNZKtsYf
</commit_message>
<xml_diff>
--- a/cartera-mixtos/data/DATOS_MIXTOS.xlsx
+++ b/cartera-mixtos/data/DATOS_MIXTOS.xlsx
@@ -1029,7 +1029,7 @@
     <t>101.7 MW / 305.1 MWh</t>
   </si>
   <si>
-    <t>$381,545,675.00</t>
+    <t>$925,310,833.00</t>
   </si>
   <si>
     <t>CONCEPCIÓN MENDIZÁBAL MENDOZA FASE II</t>
@@ -1041,13 +1041,13 @@
     <t>54 MW / 162 MWh</t>
   </si>
   <si>
-    <t>$198,977,154.00</t>
+    <t>$925,310,833.00</t>
   </si>
   <si>
     <t>CONCEPCIÓN MENDIZÁBAL MENDOZA FASE III</t>
   </si>
   <si>
-    <t>$376,737,492.00</t>
+    <t>$925,310,833.00</t>
   </si>
   <si>
     <t>35.00%</t>

</xml_diff>

<commit_message>
Mixtos: CAPEX de Concepción Mendizábal solo en la Fase II
El CAPEX único de las tres fases ($925,310,833.00) queda en la Fase II;
las fases I y III dicen "VER FASE II" (no suman en el total). Se quita
la regla de CAPEX repetido del Resumen, que ya no hace falta.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01APiq7bAy76yveceNZKtsYf
</commit_message>
<xml_diff>
--- a/cartera-mixtos/data/DATOS_MIXTOS.xlsx
+++ b/cartera-mixtos/data/DATOS_MIXTOS.xlsx
@@ -1029,25 +1029,25 @@
     <t>101.7 MW / 305.1 MWh</t>
   </si>
   <si>
+    <t>VER FASE II</t>
+  </si>
+  <si>
+    <t>CONCEPCIÓN MENDIZÁBAL MENDOZA FASE II</t>
+  </si>
+  <si>
+    <t>180 MW</t>
+  </si>
+  <si>
+    <t>54 MW / 162 MWh</t>
+  </si>
+  <si>
     <t>$925,310,833.00</t>
   </si>
   <si>
-    <t>CONCEPCIÓN MENDIZÁBAL MENDOZA FASE II</t>
-  </si>
-  <si>
-    <t>180 MW</t>
-  </si>
-  <si>
-    <t>54 MW / 162 MWh</t>
-  </si>
-  <si>
-    <t>$925,310,833.00</t>
-  </si>
-  <si>
     <t>CONCEPCIÓN MENDIZÁBAL MENDOZA FASE III</t>
   </si>
   <si>
-    <t>$925,310,833.00</t>
+    <t>VER FASE II</t>
   </si>
   <si>
     <t>35.00%</t>

</xml_diff>